<commit_message>
UFC CACE separada no modelo (premio R$ 85 mil, obra R$ 7,2 mi, honorario como % da obra)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpMcBDEADLWoT4jSWTrqdN
</commit_message>
<xml_diff>
--- a/concursos/PROJECAO_CONCURSOS_2026_2028.xlsx
+++ b/concursos/PROJECAO_CONCURSOS_2026_2028.xlsx
@@ -939,7 +939,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• A aba Monte Carlo é FIXA (20 mil rodadas por cenário). Se você mudar as premissas, peça para rodar de novo.</t>
+          <t>• A aba Monte Carlo é FIXA (200 mil rodadas por cenário). Se você mudar as premissas, peça para rodar de novo.</t>
         </is>
       </c>
     </row>
@@ -1069,151 +1069,170 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Contratos esperados ganhos (nº)</t>
-        </is>
-      </c>
-      <c r="B8" s="9">
-        <f>'Conservador'!L14</f>
-        <v/>
-      </c>
-      <c r="C8" s="9">
-        <f>'Realista'!L14</f>
-        <v/>
-      </c>
-      <c r="D8" s="9">
-        <f>'Otimista'!L14</f>
+          <t xml:space="preserve">  dos quais UFC CACE</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>'Conservador'!L44</f>
+        <v/>
+      </c>
+      <c r="C8" s="8">
+        <f>'Realista'!L44</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>'Otimista'!L44</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Contratos recebidos até dez/2028 (sua parte, bruto de imposto)</t>
-        </is>
-      </c>
-      <c r="B9" s="8">
-        <f>'Conservador'!L26</f>
-        <v/>
-      </c>
-      <c r="C9" s="8">
-        <f>'Realista'!L26</f>
-        <v/>
-      </c>
-      <c r="D9" s="8">
-        <f>'Otimista'!L26</f>
+          <t>Contratos esperados ganhos (nº)</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>'Conservador'!L41</f>
+        <v/>
+      </c>
+      <c r="C9" s="9">
+        <f>'Realista'!L41</f>
+        <v/>
+      </c>
+      <c r="D9" s="9">
+        <f>'Otimista'!L41</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Caixa líquido dos concursos</t>
+          <t>Contratos recebidos até dez/2028 (sua parte, bruto de imposto)</t>
         </is>
       </c>
       <c r="B10" s="8">
-        <f>'Conservador'!L31</f>
+        <f>'Conservador'!L26</f>
         <v/>
       </c>
       <c r="C10" s="8">
-        <f>'Realista'!L31</f>
+        <f>'Realista'!L26</f>
         <v/>
       </c>
       <c r="D10" s="8">
-        <f>'Otimista'!L31</f>
+        <f>'Otimista'!L26</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Líquido depois do valor das horas</t>
+          <t>Caixa líquido dos concursos</t>
         </is>
       </c>
       <c r="B11" s="8">
-        <f>'Conservador'!L33</f>
+        <f>'Conservador'!L31</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>'Realista'!L33</f>
+        <f>'Realista'!L31</f>
         <v/>
       </c>
       <c r="D11" s="8">
-        <f>'Otimista'!L33</f>
+        <f>'Otimista'!L31</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Líquido depois do valor das horas</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>'Conservador'!L33</f>
+        <v/>
+      </c>
+      <c r="C12" s="8">
+        <f>'Realista'!L33</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>'Otimista'!L33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Perna 2 (PSCIP/Revit/casa)</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B13" s="8">
         <f>'Conservador'!L35</f>
         <v/>
       </c>
-      <c r="C12" s="8">
+      <c r="C13" s="8">
         <f>'Realista'!L35</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D13" s="8">
         <f>'Otimista'!L35</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>RENDA TOTAL no período</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B14" s="11">
         <f>'Conservador'!L36</f>
         <v/>
       </c>
-      <c r="C13" s="11">
+      <c r="C14" s="11">
         <f>'Realista'!L36</f>
         <v/>
       </c>
-      <c r="D13" s="11">
+      <c r="D14" s="11">
         <f>'Otimista'!L36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Renda mensal média no período</t>
-        </is>
-      </c>
-      <c r="B14" s="8">
-        <f>'Conservador'!L37</f>
-        <v/>
-      </c>
-      <c r="C14" s="8">
-        <f>'Realista'!L37</f>
-        <v/>
-      </c>
-      <c r="D14" s="8">
-        <f>'Otimista'!L37</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Renda mensal média no período</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>'Conservador'!L37</f>
+        <v/>
+      </c>
+      <c r="C15" s="8">
+        <f>'Realista'!L37</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>'Otimista'!L37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Carteira de contratos ganhos a receber DEPOIS de 2028 (líquido)</t>
         </is>
       </c>
-      <c r="B15" s="8">
+      <c r="B16" s="8">
         <f>'Conservador'!L42</f>
         <v/>
       </c>
-      <c r="C15" s="8">
+      <c r="C16" s="8">
         <f>'Realista'!L42</f>
         <v/>
       </c>
-      <c r="D15" s="8">
+      <c r="D16" s="8">
         <f>'Otimista'!L42</f>
         <v/>
       </c>
@@ -1704,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -2050,59 +2069,59 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Margem sobre o honorário (depois de equipe/terceiros)</t>
+          <t>UFC CACE — prêmio do 1º lugar</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>0.55</v>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>85000</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>85000</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>85000</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Chute.</t>
+          <t>Dado seu: R$ 85 mil.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sua parte do contrato (divisão com a JOJO/sócios)</t>
+          <t>UFC CACE — valor da obra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E17" s="13" t="n">
-        <v>0.7</v>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>7200000</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>7200000</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>7200000</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Chute. Na planilha antiga estava 100%, o que superestima.</t>
+          <t>Dado seu: R$ 7,2 mi.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Imposto sobre prêmios</t>
+          <t>UFC CACE — honorário do projeto como % da obra</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2111,24 +2130,24 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Chute. Confirme com contador.</t>
+          <t>CHUTE. Projeto completo (arq + complementares) costuma ficar em 4–6% da obra. Confira o edital.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Imposto sobre contratos</t>
+          <t>Margem sobre o honorário (depois de equipe/terceiros)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2137,102 +2156,102 @@
         </is>
       </c>
       <c r="C19" s="13" t="n">
-        <v>0.16</v>
+        <v>0.55</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>0.16</v>
+        <v>0.55</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>0.16</v>
+        <v>0.55</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Chute (Simples/Lucro presumido).</t>
+          <t>Chute.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Horas por concurso nacional grande</t>
+          <t>Sua parte do contrato (divisão com a JOJO/sócios)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D20" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="E20" s="16" t="n">
-        <v>100</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>0.7</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Faixa que dei antes: 60–120 h.</t>
+          <t>Chute. Na planilha antiga estava 100%, o que superestima.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Horas por concurso internacional</t>
+          <t>Imposto sobre prêmios</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="C21" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="D21" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="E21" s="16" t="n">
-        <v>70</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>0.15</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Estimativa.</t>
+          <t>Chute. Confirme com contador.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Horas de execução de um contrato (anteprojeto→executivo)</t>
+          <t>Imposto sobre contratos</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D22" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E22" s="16" t="n">
-        <v>1200</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>0.16</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Chute. Pesa na capacidade em 2028.</t>
+          <t>Chute (Simples/Lucro presumido).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Teto de horas por trimestre (concurso + contrato)</t>
+          <t>Horas por concurso nacional grande</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2241,128 +2260,128 @@
         </is>
       </c>
       <c r="C23" s="16" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>160 h/mês, o teto que usei na planilha.</t>
+          <t>Faixa que dei antes: 60–120 h.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Valor da sua hora (custo de oportunidade)</t>
+          <t>Horas por concurso internacional</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R$/h</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="E24" s="14" t="n">
-        <v>120</v>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>70</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>70</v>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>70</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>A mesma R$ 120/h da planilha anterior.</t>
+          <t>Estimativa.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ferramentas (Claude, Magnific, licenças)</t>
+          <t>Horas de execução de um contrato (anteprojeto→executivo)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R$/mês</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D25" s="14" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E25" s="14" t="n">
-        <v>2500</v>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>1200</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Faixa que dei antes: R$ 1,5–4 mil/mês.</t>
+          <t>Chute. Pesa na capacidade em 2028.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Parte das ferramentas atribuída aos concursos</t>
+          <t>Teto de horas por trimestre (concurso + contrato)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D26" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E26" s="13" t="n">
-        <v>0.6</v>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>480</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>480</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <v>480</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Chute. O resto serve à perna 2 e a outros trabalhos.</t>
+          <t>160 h/mês, o teto que usei na planilha.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Inscrição média de concurso internacional</t>
+          <t>Valor da sua hora (custo de oportunidade)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R$</t>
+          <t>R$/h</t>
         </is>
       </c>
       <c r="C27" s="14" t="n">
-        <v>620</v>
+        <v>120</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>620</v>
+        <v>120</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>620</v>
+        <v>120</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>≈ € 100 × câmbio.</t>
+          <t>A mesma R$ 120/h da planilha anterior.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CNPJ + contabilidade (a partir de T1/27)</t>
+          <t>Ferramentas (Claude, Magnific, licenças)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2371,119 +2390,197 @@
         </is>
       </c>
       <c r="C28" s="14" t="n">
-        <v>600</v>
+        <v>2500</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>600</v>
+        <v>2500</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>600</v>
+        <v>2500</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Chute. Assume o CNPJ aberto até dez/2026.</t>
+          <t>Faixa que dei antes: R$ 1,5–4 mil/mês.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Renda mensal da 'perna 2' (PSCIP/PICIP, Revit, casa)</t>
+          <t>Parte das ferramentas atribuída aos concursos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R$/mês</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="n">
-        <v>6000</v>
-      </c>
-      <c r="D29" s="14" t="n">
-        <v>7000</v>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>8000</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>0.6</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CHUTE TOTAL. Troque pelo seu número real.</t>
+          <t>Chute. O resto serve à perna 2 e a outros trabalhos.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Crescimento anual da perna 2</t>
+          <t>Inscrição média de concurso internacional</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>0.12</v>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>620</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>620</v>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>620</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Chute.</t>
+          <t>≈ € 100 × câmbio.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Alta da perna 2 após ganhar autoridade (menção/1º)</t>
+          <t>CNPJ + contabilidade (a partir de T1/27)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E31" s="13" t="n">
-        <v>0.3</v>
+          <t>R$/mês</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>600</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>600</v>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>600</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Cliente privado paga mais depois de prêmio. Chute.</t>
+          <t>Chute. Assume o CNPJ aberto até dez/2026.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Renda mensal da 'perna 2' (PSCIP/PICIP, Revit, casa)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>R$/mês</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>CHUTE TOTAL. Troque pelo seu número real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Crescimento anual da perna 2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E33" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Chute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Alta da perna 2 após ganhar autoridade (menção/1º)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Cliente privado paga mais depois de prêmio. Chute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Trimestre (nº) em que a alta começa (1=T4/26 … 9=T4/28)</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>nº</t>
         </is>
       </c>
-      <c r="C32" s="16" t="n">
+      <c r="C35" s="16" t="n">
         <v>99</v>
       </c>
-      <c r="D32" s="16" t="n">
+      <c r="D35" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E32" s="16" t="n">
+      <c r="E35" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>99 = nunca acontece.</t>
         </is>
@@ -2500,7 +2597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2650,7 +2747,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Concursos nacionais grandes inscritos</t>
+          <t>Concursos nacionais grandes inscritos (sem a UFC; a UFC está em T4/26 à parte)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2659,7 +2756,7 @@
         </is>
       </c>
       <c r="C7" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>0</v>
@@ -2865,39 +2962,39 @@
         </is>
       </c>
       <c r="C12" s="8">
-        <f>C10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>C10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+C44</f>
         <v/>
       </c>
       <c r="D12" s="8">
-        <f>D10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>D10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+D44</f>
         <v/>
       </c>
       <c r="E12" s="8">
-        <f>E10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>E10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+E44</f>
         <v/>
       </c>
       <c r="F12" s="8">
-        <f>F10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>F10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+F44</f>
         <v/>
       </c>
       <c r="G12" s="8">
-        <f>G10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>G10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+G44</f>
         <v/>
       </c>
       <c r="H12" s="8">
-        <f>H10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>H10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+H44</f>
         <v/>
       </c>
       <c r="I12" s="8">
-        <f>I10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>I10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+I44</f>
         <v/>
       </c>
       <c r="J12" s="8">
-        <f>J10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>J10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+J44</f>
         <v/>
       </c>
       <c r="K12" s="8">
-        <f>K10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)</f>
+        <f>K10*(Premissas!$C$6*Premissas!$C$10+Premissas!$C$7*Premissas!$C$11)+K44</f>
         <v/>
       </c>
       <c r="L12" s="23">
@@ -3039,39 +3136,39 @@
         </is>
       </c>
       <c r="C16" s="8">
-        <f>Premissas!$C$15/4*0</f>
+        <f>Premissas!$C$15/4*0+C46</f>
         <v/>
       </c>
       <c r="D16" s="8">
-        <f>Premissas!$C$15/4*0</f>
+        <f>Premissas!$C$15/4*0+D46</f>
         <v/>
       </c>
       <c r="E16" s="8">
-        <f>Premissas!$C$15/4*0</f>
+        <f>Premissas!$C$15/4*0+E46</f>
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>Premissas!$C$15/4*SUM(C14:C14)</f>
+        <f>Premissas!$C$15/4*SUM(C14:C14)+F46</f>
         <v/>
       </c>
       <c r="G16" s="8">
-        <f>Premissas!$C$15/4*SUM(C14:D14)</f>
+        <f>Premissas!$C$15/4*SUM(C14:D14)+G46</f>
         <v/>
       </c>
       <c r="H16" s="8">
-        <f>Premissas!$C$15/4*SUM(C14:E14)</f>
+        <f>Premissas!$C$15/4*SUM(C14:E14)+H46</f>
         <v/>
       </c>
       <c r="I16" s="8">
-        <f>Premissas!$C$15/4*SUM(C14:F14)</f>
+        <f>Premissas!$C$15/4*SUM(C14:F14)+I46</f>
         <v/>
       </c>
       <c r="J16" s="8">
-        <f>Premissas!$C$15/4*SUM(D14:G14)</f>
+        <f>Premissas!$C$15/4*SUM(D14:G14)+J46</f>
         <v/>
       </c>
       <c r="K16" s="8">
-        <f>Premissas!$C$15/4*SUM(E14:H14)</f>
+        <f>Premissas!$C$15/4*SUM(E14:H14)+K46</f>
         <v/>
       </c>
       <c r="L16" s="23">
@@ -3091,39 +3188,39 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>C16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>C16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>D16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>D16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>E16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>E16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>F16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>F16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>G16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>G16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>H16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>H16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>I16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>I16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="J17" s="8">
-        <f>J16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>J16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="K17" s="8">
-        <f>K16*Premissas!$C$16*Premissas!$C$17</f>
+        <f>K16*Premissas!$C$19*Premissas!$C$20</f>
         <v/>
       </c>
       <c r="L17" s="23">
@@ -3143,39 +3240,39 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>Premissas!$C$22/4*0</f>
+        <f>Premissas!$C$25/4*0+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="D18" s="7">
-        <f>Premissas!$C$22/4*0</f>
+        <f>Premissas!$C$25/4*0+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>Premissas!$C$22/4*0</f>
+        <f>Premissas!$C$25/4*0+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>Premissas!$C$22/4*SUM(C14:C14)</f>
+        <f>Premissas!$C$25/4*SUM(C14:C14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>Premissas!$C$22/4*SUM(C14:D14)</f>
+        <f>Premissas!$C$25/4*SUM(C14:D14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>Premissas!$C$22/4*SUM(C14:E14)</f>
+        <f>Premissas!$C$25/4*SUM(C14:E14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>Premissas!$C$22/4*SUM(C14:F14)</f>
+        <f>Premissas!$C$25/4*SUM(C14:F14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="J18" s="7">
-        <f>Premissas!$C$22/4*SUM(D14:G14)</f>
+        <f>Premissas!$C$25/4*SUM(D14:G14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>Premissas!$C$22/4*SUM(E14:H14)</f>
+        <f>Premissas!$C$25/4*SUM(E14:H14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -3213,39 +3310,39 @@
         </is>
       </c>
       <c r="C20" s="7">
-        <f>C7*Premissas!$C$20+C8*Premissas!$C$21</f>
+        <f>C7*Premissas!$C$23+C8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="D20" s="7">
-        <f>D7*Premissas!$C$20+D8*Premissas!$C$21</f>
+        <f>D7*Premissas!$C$23+D8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>E7*Premissas!$C$20+E8*Premissas!$C$21</f>
+        <f>E7*Premissas!$C$23+E8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>F7*Premissas!$C$20+F8*Premissas!$C$21</f>
+        <f>F7*Premissas!$C$23+F8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>G7*Premissas!$C$20+G8*Premissas!$C$21</f>
+        <f>G7*Premissas!$C$23+G8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>H7*Premissas!$C$20+H8*Premissas!$C$21</f>
+        <f>H7*Premissas!$C$23+H8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>I7*Premissas!$C$20+I8*Premissas!$C$21</f>
+        <f>I7*Premissas!$C$23+I8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="J20" s="7">
-        <f>J7*Premissas!$C$20+J8*Premissas!$C$21</f>
+        <f>J7*Premissas!$C$23+J8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>K7*Premissas!$C$20+K8*Premissas!$C$21</f>
+        <f>K7*Premissas!$C$23+K8*Premissas!$C$24</f>
         <v/>
       </c>
       <c r="L20" s="22">
@@ -3314,39 +3411,39 @@
         </is>
       </c>
       <c r="C22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="D22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="J22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>Premissas!$C$23</f>
+        <f>Premissas!$C$26</f>
         <v/>
       </c>
       <c r="L22" s="7" t="n"/>
@@ -3530,39 +3627,39 @@
         </is>
       </c>
       <c r="C27" s="8">
-        <f>-(C25*Premissas!$C$18+C26*Premissas!$C$19)</f>
+        <f>-(C25*Premissas!$C$21+C26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>-(D25*Premissas!$C$18+D26*Premissas!$C$19)</f>
+        <f>-(D25*Premissas!$C$21+D26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>-(E25*Premissas!$C$18+E26*Premissas!$C$19)</f>
+        <f>-(E25*Premissas!$C$21+E26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>-(F25*Premissas!$C$18+F26*Premissas!$C$19)</f>
+        <f>-(F25*Premissas!$C$21+F26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="G27" s="8">
-        <f>-(G25*Premissas!$C$18+G26*Premissas!$C$19)</f>
+        <f>-(G25*Premissas!$C$21+G26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="H27" s="8">
-        <f>-(H25*Premissas!$C$18+H26*Premissas!$C$19)</f>
+        <f>-(H25*Premissas!$C$21+H26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="I27" s="8">
-        <f>-(I25*Premissas!$C$18+I26*Premissas!$C$19)</f>
+        <f>-(I25*Premissas!$C$21+I26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>-(J25*Premissas!$C$18+J26*Premissas!$C$19)</f>
+        <f>-(J25*Premissas!$C$21+J26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="K27" s="8">
-        <f>-(K25*Premissas!$C$18+K26*Premissas!$C$19)</f>
+        <f>-(K25*Premissas!$C$21+K26*Premissas!$C$22)</f>
         <v/>
       </c>
       <c r="L27" s="23">
@@ -3582,39 +3679,39 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="G28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="H28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="I28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="J28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="K28" s="8">
-        <f>-3*Premissas!$C$25*Premissas!$C$26</f>
+        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
         <v/>
       </c>
       <c r="L28" s="23">
@@ -3634,39 +3731,39 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>-C8*Premissas!$C$27</f>
+        <f>-C8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>-D8*Premissas!$C$27</f>
+        <f>-D8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>-E8*Premissas!$C$27</f>
+        <f>-E8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>-F8*Premissas!$C$27</f>
+        <f>-F8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>-G8*Premissas!$C$27</f>
+        <f>-G8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>-H8*Premissas!$C$27</f>
+        <f>-H8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>-I8*Premissas!$C$27</f>
+        <f>-I8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>-J8*Premissas!$C$27</f>
+        <f>-J8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>-K8*Premissas!$C$27</f>
+        <f>-K8*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="L29" s="23">
@@ -3689,35 +3786,35 @@
         <v>0</v>
       </c>
       <c r="D30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="G30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="H30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="I30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="J30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="K30" s="8">
-        <f>-3*Premissas!$C$28</f>
+        <f>-3*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="L30" s="23">
@@ -3789,39 +3886,39 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>-C20*Premissas!$C$24</f>
+        <f>-C20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="D32" s="8">
-        <f>-D20*Premissas!$C$24</f>
+        <f>-D20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="E32" s="8">
-        <f>-E20*Premissas!$C$24</f>
+        <f>-E20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="F32" s="8">
-        <f>-F20*Premissas!$C$24</f>
+        <f>-F20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="G32" s="8">
-        <f>-G20*Premissas!$C$24</f>
+        <f>-G20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="H32" s="8">
-        <f>-H20*Premissas!$C$24</f>
+        <f>-H20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="I32" s="8">
-        <f>-I20*Premissas!$C$24</f>
+        <f>-I20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="J32" s="8">
-        <f>-J20*Premissas!$C$24</f>
+        <f>-J20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="K32" s="8">
-        <f>-K20*Premissas!$C$24</f>
+        <f>-K20*Premissas!$C$27</f>
         <v/>
       </c>
       <c r="L32" s="23">
@@ -3911,39 +4008,39 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="H35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="I35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="J35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="K35" s="8">
-        <f>3*Premissas!$C$29*(1+Premissas!$C$30)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$C$32,Premissas!$C$31,0))</f>
+        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
         <v/>
       </c>
       <c r="L35" s="23">
@@ -4192,7 +4289,7 @@
       <c r="J41" s="9" t="n"/>
       <c r="K41" s="9" t="n"/>
       <c r="L41" s="24">
-        <f>L14</f>
+        <f>L14+L45</f>
         <v/>
       </c>
     </row>
@@ -4217,7 +4314,160 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="23">
-        <f>L14*Premissas!$C$15*Premissas!$C$16*Premissas!$C$17*(1-Premissas!$C$19)-L26*(1-Premissas!$C$19)</f>
+        <f>(L14*Premissas!$C$15+L45*Premissas!$C$17*Premissas!$C$18)*Premissas!$C$19*Premissas!$C$20*(1-Premissas!$C$22)-L26*(1-Premissas!$C$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>UFC CACE (entrega 21/10/2026, resultado em T1/27) — separado do genérico</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+      <c r="J43" s="20" t="n"/>
+      <c r="K43" s="20" t="n"/>
+      <c r="L43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UFC: prêmio esperado (1º ou menção)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="8">
+        <f>Premissas!$C$6*Premissas!$C$16+Premissas!$C$7*Premissas!$C$11</f>
+        <v/>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="23">
+        <f>SUM(C44:K44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UFC: contrato esperado ganho (nº)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>nº</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="9">
+        <f>Premissas!$C$6*Premissas!$C$14</f>
+        <v/>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="24">
+        <f>SUM(C45:K45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UFC: honorário bruto recebido pelo escritório</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="8">
+        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="H46" s="8">
+        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="I46" s="8">
+        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="J46" s="8">
+        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="K46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="23">
+        <f>SUM(C46:K46)</f>
         <v/>
       </c>
     </row>
@@ -4232,7 +4482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -4382,7 +4632,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Concursos nacionais grandes inscritos</t>
+          <t>Concursos nacionais grandes inscritos (sem a UFC; a UFC está em T4/26 à parte)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4391,7 +4641,7 @@
         </is>
       </c>
       <c r="C7" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>1</v>
@@ -4597,39 +4847,39 @@
         </is>
       </c>
       <c r="C12" s="8">
-        <f>C10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>C10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+C44</f>
         <v/>
       </c>
       <c r="D12" s="8">
-        <f>D10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>D10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+D44</f>
         <v/>
       </c>
       <c r="E12" s="8">
-        <f>E10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>E10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+E44</f>
         <v/>
       </c>
       <c r="F12" s="8">
-        <f>F10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>F10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+F44</f>
         <v/>
       </c>
       <c r="G12" s="8">
-        <f>G10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>G10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+G44</f>
         <v/>
       </c>
       <c r="H12" s="8">
-        <f>H10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>H10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+H44</f>
         <v/>
       </c>
       <c r="I12" s="8">
-        <f>I10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>I10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+I44</f>
         <v/>
       </c>
       <c r="J12" s="8">
-        <f>J10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>J10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+J44</f>
         <v/>
       </c>
       <c r="K12" s="8">
-        <f>K10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)</f>
+        <f>K10*(Premissas!$D$6*Premissas!$D$10+Premissas!$D$7*Premissas!$D$11)+K44</f>
         <v/>
       </c>
       <c r="L12" s="23">
@@ -4771,39 +5021,39 @@
         </is>
       </c>
       <c r="C16" s="8">
-        <f>Premissas!$D$15/4*0</f>
+        <f>Premissas!$D$15/4*0+C46</f>
         <v/>
       </c>
       <c r="D16" s="8">
-        <f>Premissas!$D$15/4*0</f>
+        <f>Premissas!$D$15/4*0+D46</f>
         <v/>
       </c>
       <c r="E16" s="8">
-        <f>Premissas!$D$15/4*0</f>
+        <f>Premissas!$D$15/4*0+E46</f>
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>Premissas!$D$15/4*SUM(C14:C14)</f>
+        <f>Premissas!$D$15/4*SUM(C14:C14)+F46</f>
         <v/>
       </c>
       <c r="G16" s="8">
-        <f>Premissas!$D$15/4*SUM(C14:D14)</f>
+        <f>Premissas!$D$15/4*SUM(C14:D14)+G46</f>
         <v/>
       </c>
       <c r="H16" s="8">
-        <f>Premissas!$D$15/4*SUM(C14:E14)</f>
+        <f>Premissas!$D$15/4*SUM(C14:E14)+H46</f>
         <v/>
       </c>
       <c r="I16" s="8">
-        <f>Premissas!$D$15/4*SUM(C14:F14)</f>
+        <f>Premissas!$D$15/4*SUM(C14:F14)+I46</f>
         <v/>
       </c>
       <c r="J16" s="8">
-        <f>Premissas!$D$15/4*SUM(D14:G14)</f>
+        <f>Premissas!$D$15/4*SUM(D14:G14)+J46</f>
         <v/>
       </c>
       <c r="K16" s="8">
-        <f>Premissas!$D$15/4*SUM(E14:H14)</f>
+        <f>Premissas!$D$15/4*SUM(E14:H14)+K46</f>
         <v/>
       </c>
       <c r="L16" s="23">
@@ -4823,39 +5073,39 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>C16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>C16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>D16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>D16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>E16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>E16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>F16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>F16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>G16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>G16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>H16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>H16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>I16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>I16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="J17" s="8">
-        <f>J16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>J16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="K17" s="8">
-        <f>K16*Premissas!$D$16*Premissas!$D$17</f>
+        <f>K16*Premissas!$D$19*Premissas!$D$20</f>
         <v/>
       </c>
       <c r="L17" s="23">
@@ -4875,39 +5125,39 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>Premissas!$D$22/4*0</f>
+        <f>Premissas!$D$25/4*0+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="D18" s="7">
-        <f>Premissas!$D$22/4*0</f>
+        <f>Premissas!$D$25/4*0+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>Premissas!$D$22/4*0</f>
+        <f>Premissas!$D$25/4*0+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>Premissas!$D$22/4*SUM(C14:C14)</f>
+        <f>Premissas!$D$25/4*SUM(C14:C14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>Premissas!$D$22/4*SUM(C14:D14)</f>
+        <f>Premissas!$D$25/4*SUM(C14:D14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>Premissas!$D$22/4*SUM(C14:E14)</f>
+        <f>Premissas!$D$25/4*SUM(C14:E14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>Premissas!$D$22/4*SUM(C14:F14)</f>
+        <f>Premissas!$D$25/4*SUM(C14:F14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="J18" s="7">
-        <f>Premissas!$D$22/4*SUM(D14:G14)</f>
+        <f>Premissas!$D$25/4*SUM(D14:G14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>Premissas!$D$22/4*SUM(E14:H14)</f>
+        <f>Premissas!$D$25/4*SUM(E14:H14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -4945,39 +5195,39 @@
         </is>
       </c>
       <c r="C20" s="7">
-        <f>C7*Premissas!$D$20+C8*Premissas!$D$21</f>
+        <f>C7*Premissas!$D$23+C8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="D20" s="7">
-        <f>D7*Premissas!$D$20+D8*Premissas!$D$21</f>
+        <f>D7*Premissas!$D$23+D8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>E7*Premissas!$D$20+E8*Premissas!$D$21</f>
+        <f>E7*Premissas!$D$23+E8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>F7*Premissas!$D$20+F8*Premissas!$D$21</f>
+        <f>F7*Premissas!$D$23+F8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>G7*Premissas!$D$20+G8*Premissas!$D$21</f>
+        <f>G7*Premissas!$D$23+G8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>H7*Premissas!$D$20+H8*Premissas!$D$21</f>
+        <f>H7*Premissas!$D$23+H8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>I7*Premissas!$D$20+I8*Premissas!$D$21</f>
+        <f>I7*Premissas!$D$23+I8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="J20" s="7">
-        <f>J7*Premissas!$D$20+J8*Premissas!$D$21</f>
+        <f>J7*Premissas!$D$23+J8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>K7*Premissas!$D$20+K8*Premissas!$D$21</f>
+        <f>K7*Premissas!$D$23+K8*Premissas!$D$24</f>
         <v/>
       </c>
       <c r="L20" s="22">
@@ -5046,39 +5296,39 @@
         </is>
       </c>
       <c r="C22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="D22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="J22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>Premissas!$D$23</f>
+        <f>Premissas!$D$26</f>
         <v/>
       </c>
       <c r="L22" s="7" t="n"/>
@@ -5262,39 +5512,39 @@
         </is>
       </c>
       <c r="C27" s="8">
-        <f>-(C25*Premissas!$D$18+C26*Premissas!$D$19)</f>
+        <f>-(C25*Premissas!$D$21+C26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>-(D25*Premissas!$D$18+D26*Premissas!$D$19)</f>
+        <f>-(D25*Premissas!$D$21+D26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>-(E25*Premissas!$D$18+E26*Premissas!$D$19)</f>
+        <f>-(E25*Premissas!$D$21+E26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>-(F25*Premissas!$D$18+F26*Premissas!$D$19)</f>
+        <f>-(F25*Premissas!$D$21+F26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="G27" s="8">
-        <f>-(G25*Premissas!$D$18+G26*Premissas!$D$19)</f>
+        <f>-(G25*Premissas!$D$21+G26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="H27" s="8">
-        <f>-(H25*Premissas!$D$18+H26*Premissas!$D$19)</f>
+        <f>-(H25*Premissas!$D$21+H26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="I27" s="8">
-        <f>-(I25*Premissas!$D$18+I26*Premissas!$D$19)</f>
+        <f>-(I25*Premissas!$D$21+I26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>-(J25*Premissas!$D$18+J26*Premissas!$D$19)</f>
+        <f>-(J25*Premissas!$D$21+J26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="K27" s="8">
-        <f>-(K25*Premissas!$D$18+K26*Premissas!$D$19)</f>
+        <f>-(K25*Premissas!$D$21+K26*Premissas!$D$22)</f>
         <v/>
       </c>
       <c r="L27" s="23">
@@ -5314,39 +5564,39 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="G28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="H28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="I28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="J28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="K28" s="8">
-        <f>-3*Premissas!$D$25*Premissas!$D$26</f>
+        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
         <v/>
       </c>
       <c r="L28" s="23">
@@ -5366,39 +5616,39 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>-C8*Premissas!$D$27</f>
+        <f>-C8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>-D8*Premissas!$D$27</f>
+        <f>-D8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>-E8*Premissas!$D$27</f>
+        <f>-E8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>-F8*Premissas!$D$27</f>
+        <f>-F8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>-G8*Premissas!$D$27</f>
+        <f>-G8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>-H8*Premissas!$D$27</f>
+        <f>-H8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>-I8*Premissas!$D$27</f>
+        <f>-I8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>-J8*Premissas!$D$27</f>
+        <f>-J8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>-K8*Premissas!$D$27</f>
+        <f>-K8*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="L29" s="23">
@@ -5421,35 +5671,35 @@
         <v>0</v>
       </c>
       <c r="D30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="G30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="H30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="I30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="J30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="K30" s="8">
-        <f>-3*Premissas!$D$28</f>
+        <f>-3*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="L30" s="23">
@@ -5521,39 +5771,39 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>-C20*Premissas!$D$24</f>
+        <f>-C20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="D32" s="8">
-        <f>-D20*Premissas!$D$24</f>
+        <f>-D20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="E32" s="8">
-        <f>-E20*Premissas!$D$24</f>
+        <f>-E20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="F32" s="8">
-        <f>-F20*Premissas!$D$24</f>
+        <f>-F20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="G32" s="8">
-        <f>-G20*Premissas!$D$24</f>
+        <f>-G20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="H32" s="8">
-        <f>-H20*Premissas!$D$24</f>
+        <f>-H20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="I32" s="8">
-        <f>-I20*Premissas!$D$24</f>
+        <f>-I20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="J32" s="8">
-        <f>-J20*Premissas!$D$24</f>
+        <f>-J20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="K32" s="8">
-        <f>-K20*Premissas!$D$24</f>
+        <f>-K20*Premissas!$D$27</f>
         <v/>
       </c>
       <c r="L32" s="23">
@@ -5643,39 +5893,39 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="H35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="I35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="J35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="K35" s="8">
-        <f>3*Premissas!$D$29*(1+Premissas!$D$30)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$D$32,Premissas!$D$31,0))</f>
+        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
         <v/>
       </c>
       <c r="L35" s="23">
@@ -5924,7 +6174,7 @@
       <c r="J41" s="9" t="n"/>
       <c r="K41" s="9" t="n"/>
       <c r="L41" s="24">
-        <f>L14</f>
+        <f>L14+L45</f>
         <v/>
       </c>
     </row>
@@ -5949,7 +6199,160 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="23">
-        <f>L14*Premissas!$D$15*Premissas!$D$16*Premissas!$D$17*(1-Premissas!$D$19)-L26*(1-Premissas!$D$19)</f>
+        <f>(L14*Premissas!$D$15+L45*Premissas!$D$17*Premissas!$D$18)*Premissas!$D$19*Premissas!$D$20*(1-Premissas!$D$22)-L26*(1-Premissas!$D$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>UFC CACE (entrega 21/10/2026, resultado em T1/27) — separado do genérico</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+      <c r="J43" s="20" t="n"/>
+      <c r="K43" s="20" t="n"/>
+      <c r="L43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UFC: prêmio esperado (1º ou menção)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="8">
+        <f>Premissas!$D$6*Premissas!$D$16+Premissas!$D$7*Premissas!$D$11</f>
+        <v/>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="23">
+        <f>SUM(C44:K44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UFC: contrato esperado ganho (nº)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>nº</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="9">
+        <f>Premissas!$D$6*Premissas!$D$14</f>
+        <v/>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="24">
+        <f>SUM(C45:K45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UFC: honorário bruto recebido pelo escritório</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="8">
+        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="H46" s="8">
+        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="I46" s="8">
+        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="J46" s="8">
+        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="K46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="23">
+        <f>SUM(C46:K46)</f>
         <v/>
       </c>
     </row>
@@ -5964,7 +6367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -6114,7 +6517,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Concursos nacionais grandes inscritos</t>
+          <t>Concursos nacionais grandes inscritos (sem a UFC; a UFC está em T4/26 à parte)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6123,7 +6526,7 @@
         </is>
       </c>
       <c r="C7" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>2</v>
@@ -6329,39 +6732,39 @@
         </is>
       </c>
       <c r="C12" s="8">
-        <f>C10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>C10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+C44</f>
         <v/>
       </c>
       <c r="D12" s="8">
-        <f>D10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>D10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+D44</f>
         <v/>
       </c>
       <c r="E12" s="8">
-        <f>E10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>E10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+E44</f>
         <v/>
       </c>
       <c r="F12" s="8">
-        <f>F10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>F10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+F44</f>
         <v/>
       </c>
       <c r="G12" s="8">
-        <f>G10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>G10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+G44</f>
         <v/>
       </c>
       <c r="H12" s="8">
-        <f>H10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>H10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+H44</f>
         <v/>
       </c>
       <c r="I12" s="8">
-        <f>I10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>I10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+I44</f>
         <v/>
       </c>
       <c r="J12" s="8">
-        <f>J10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>J10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+J44</f>
         <v/>
       </c>
       <c r="K12" s="8">
-        <f>K10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)</f>
+        <f>K10*(Premissas!$E$6*Premissas!$E$10+Premissas!$E$7*Premissas!$E$11)+K44</f>
         <v/>
       </c>
       <c r="L12" s="23">
@@ -6503,39 +6906,39 @@
         </is>
       </c>
       <c r="C16" s="8">
-        <f>Premissas!$E$15/4*0</f>
+        <f>Premissas!$E$15/4*0+C46</f>
         <v/>
       </c>
       <c r="D16" s="8">
-        <f>Premissas!$E$15/4*0</f>
+        <f>Premissas!$E$15/4*0+D46</f>
         <v/>
       </c>
       <c r="E16" s="8">
-        <f>Premissas!$E$15/4*0</f>
+        <f>Premissas!$E$15/4*0+E46</f>
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>Premissas!$E$15/4*SUM(C14:C14)</f>
+        <f>Premissas!$E$15/4*SUM(C14:C14)+F46</f>
         <v/>
       </c>
       <c r="G16" s="8">
-        <f>Premissas!$E$15/4*SUM(C14:D14)</f>
+        <f>Premissas!$E$15/4*SUM(C14:D14)+G46</f>
         <v/>
       </c>
       <c r="H16" s="8">
-        <f>Premissas!$E$15/4*SUM(C14:E14)</f>
+        <f>Premissas!$E$15/4*SUM(C14:E14)+H46</f>
         <v/>
       </c>
       <c r="I16" s="8">
-        <f>Premissas!$E$15/4*SUM(C14:F14)</f>
+        <f>Premissas!$E$15/4*SUM(C14:F14)+I46</f>
         <v/>
       </c>
       <c r="J16" s="8">
-        <f>Premissas!$E$15/4*SUM(D14:G14)</f>
+        <f>Premissas!$E$15/4*SUM(D14:G14)+J46</f>
         <v/>
       </c>
       <c r="K16" s="8">
-        <f>Premissas!$E$15/4*SUM(E14:H14)</f>
+        <f>Premissas!$E$15/4*SUM(E14:H14)+K46</f>
         <v/>
       </c>
       <c r="L16" s="23">
@@ -6555,39 +6958,39 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>C16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>C16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>D16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>D16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>E16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>E16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>F16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>F16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>G16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>G16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>H16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>H16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>I16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>I16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="J17" s="8">
-        <f>J16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>J16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="K17" s="8">
-        <f>K16*Premissas!$E$16*Premissas!$E$17</f>
+        <f>K16*Premissas!$E$19*Premissas!$E$20</f>
         <v/>
       </c>
       <c r="L17" s="23">
@@ -6607,39 +7010,39 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>Premissas!$E$22/4*0</f>
+        <f>Premissas!$E$25/4*0+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="D18" s="7">
-        <f>Premissas!$E$22/4*0</f>
+        <f>Premissas!$E$25/4*0+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>Premissas!$E$22/4*0</f>
+        <f>Premissas!$E$25/4*0+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>Premissas!$E$22/4*SUM(C14:C14)</f>
+        <f>Premissas!$E$25/4*SUM(C14:C14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>Premissas!$E$22/4*SUM(C14:D14)</f>
+        <f>Premissas!$E$25/4*SUM(C14:D14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>Premissas!$E$22/4*SUM(C14:E14)</f>
+        <f>Premissas!$E$25/4*SUM(C14:E14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>Premissas!$E$22/4*SUM(C14:F14)</f>
+        <f>Premissas!$E$25/4*SUM(C14:F14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="J18" s="7">
-        <f>Premissas!$E$22/4*SUM(D14:G14)</f>
+        <f>Premissas!$E$25/4*SUM(D14:G14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>Premissas!$E$22/4*SUM(E14:H14)</f>
+        <f>Premissas!$E$25/4*SUM(E14:H14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -6677,39 +7080,39 @@
         </is>
       </c>
       <c r="C20" s="7">
-        <f>C7*Premissas!$E$20+C8*Premissas!$E$21</f>
+        <f>C7*Premissas!$E$23+C8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="D20" s="7">
-        <f>D7*Premissas!$E$20+D8*Premissas!$E$21</f>
+        <f>D7*Premissas!$E$23+D8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>E7*Premissas!$E$20+E8*Premissas!$E$21</f>
+        <f>E7*Premissas!$E$23+E8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>F7*Premissas!$E$20+F8*Premissas!$E$21</f>
+        <f>F7*Premissas!$E$23+F8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>G7*Premissas!$E$20+G8*Premissas!$E$21</f>
+        <f>G7*Premissas!$E$23+G8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>H7*Premissas!$E$20+H8*Premissas!$E$21</f>
+        <f>H7*Premissas!$E$23+H8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>I7*Premissas!$E$20+I8*Premissas!$E$21</f>
+        <f>I7*Premissas!$E$23+I8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="J20" s="7">
-        <f>J7*Premissas!$E$20+J8*Premissas!$E$21</f>
+        <f>J7*Premissas!$E$23+J8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>K7*Premissas!$E$20+K8*Premissas!$E$21</f>
+        <f>K7*Premissas!$E$23+K8*Premissas!$E$24</f>
         <v/>
       </c>
       <c r="L20" s="22">
@@ -6778,39 +7181,39 @@
         </is>
       </c>
       <c r="C22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="D22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="J22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>Premissas!$E$23</f>
+        <f>Premissas!$E$26</f>
         <v/>
       </c>
       <c r="L22" s="7" t="n"/>
@@ -6994,39 +7397,39 @@
         </is>
       </c>
       <c r="C27" s="8">
-        <f>-(C25*Premissas!$E$18+C26*Premissas!$E$19)</f>
+        <f>-(C25*Premissas!$E$21+C26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>-(D25*Premissas!$E$18+D26*Premissas!$E$19)</f>
+        <f>-(D25*Premissas!$E$21+D26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>-(E25*Premissas!$E$18+E26*Premissas!$E$19)</f>
+        <f>-(E25*Premissas!$E$21+E26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>-(F25*Premissas!$E$18+F26*Premissas!$E$19)</f>
+        <f>-(F25*Premissas!$E$21+F26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="G27" s="8">
-        <f>-(G25*Premissas!$E$18+G26*Premissas!$E$19)</f>
+        <f>-(G25*Premissas!$E$21+G26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="H27" s="8">
-        <f>-(H25*Premissas!$E$18+H26*Premissas!$E$19)</f>
+        <f>-(H25*Premissas!$E$21+H26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="I27" s="8">
-        <f>-(I25*Premissas!$E$18+I26*Premissas!$E$19)</f>
+        <f>-(I25*Premissas!$E$21+I26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>-(J25*Premissas!$E$18+J26*Premissas!$E$19)</f>
+        <f>-(J25*Premissas!$E$21+J26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="K27" s="8">
-        <f>-(K25*Premissas!$E$18+K26*Premissas!$E$19)</f>
+        <f>-(K25*Premissas!$E$21+K26*Premissas!$E$22)</f>
         <v/>
       </c>
       <c r="L27" s="23">
@@ -7046,39 +7449,39 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="G28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="H28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="I28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="J28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="K28" s="8">
-        <f>-3*Premissas!$E$25*Premissas!$E$26</f>
+        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
         <v/>
       </c>
       <c r="L28" s="23">
@@ -7098,39 +7501,39 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>-C8*Premissas!$E$27</f>
+        <f>-C8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>-D8*Premissas!$E$27</f>
+        <f>-D8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>-E8*Premissas!$E$27</f>
+        <f>-E8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>-F8*Premissas!$E$27</f>
+        <f>-F8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>-G8*Premissas!$E$27</f>
+        <f>-G8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>-H8*Premissas!$E$27</f>
+        <f>-H8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>-I8*Premissas!$E$27</f>
+        <f>-I8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>-J8*Premissas!$E$27</f>
+        <f>-J8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>-K8*Premissas!$E$27</f>
+        <f>-K8*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="L29" s="23">
@@ -7153,35 +7556,35 @@
         <v>0</v>
       </c>
       <c r="D30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="G30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="H30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="I30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="J30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="K30" s="8">
-        <f>-3*Premissas!$E$28</f>
+        <f>-3*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="L30" s="23">
@@ -7253,39 +7656,39 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>-C20*Premissas!$E$24</f>
+        <f>-C20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="D32" s="8">
-        <f>-D20*Premissas!$E$24</f>
+        <f>-D20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="E32" s="8">
-        <f>-E20*Premissas!$E$24</f>
+        <f>-E20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="F32" s="8">
-        <f>-F20*Premissas!$E$24</f>
+        <f>-F20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="G32" s="8">
-        <f>-G20*Premissas!$E$24</f>
+        <f>-G20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="H32" s="8">
-        <f>-H20*Premissas!$E$24</f>
+        <f>-H20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="I32" s="8">
-        <f>-I20*Premissas!$E$24</f>
+        <f>-I20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="J32" s="8">
-        <f>-J20*Premissas!$E$24</f>
+        <f>-J20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="K32" s="8">
-        <f>-K20*Premissas!$E$24</f>
+        <f>-K20*Premissas!$E$27</f>
         <v/>
       </c>
       <c r="L32" s="23">
@@ -7375,39 +7778,39 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="H35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="I35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="J35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="K35" s="8">
-        <f>3*Premissas!$E$29*(1+Premissas!$E$30)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$E$32,Premissas!$E$31,0))</f>
+        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
         <v/>
       </c>
       <c r="L35" s="23">
@@ -7656,7 +8059,7 @@
       <c r="J41" s="9" t="n"/>
       <c r="K41" s="9" t="n"/>
       <c r="L41" s="24">
-        <f>L14</f>
+        <f>L14+L45</f>
         <v/>
       </c>
     </row>
@@ -7681,7 +8084,160 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="23">
-        <f>L14*Premissas!$E$15*Premissas!$E$16*Premissas!$E$17*(1-Premissas!$E$19)-L26*(1-Premissas!$E$19)</f>
+        <f>(L14*Premissas!$E$15+L45*Premissas!$E$17*Premissas!$E$18)*Premissas!$E$19*Premissas!$E$20*(1-Premissas!$E$22)-L26*(1-Premissas!$E$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>UFC CACE (entrega 21/10/2026, resultado em T1/27) — separado do genérico</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+      <c r="J43" s="20" t="n"/>
+      <c r="K43" s="20" t="n"/>
+      <c r="L43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UFC: prêmio esperado (1º ou menção)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="8">
+        <f>Premissas!$E$6*Premissas!$E$16+Premissas!$E$7*Premissas!$E$11</f>
+        <v/>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="23">
+        <f>SUM(C44:K44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UFC: contrato esperado ganho (nº)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>nº</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="9">
+        <f>Premissas!$E$6*Premissas!$E$14</f>
+        <v/>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="24">
+        <f>SUM(C45:K45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UFC: honorário bruto recebido pelo escritório</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="8">
+        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="H46" s="8">
+        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="I46" s="8">
+        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="J46" s="8">
+        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <v/>
+      </c>
+      <c r="K46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="23">
+        <f>SUM(C46:K46)</f>
         <v/>
       </c>
     </row>
@@ -7708,7 +8264,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>MONTE CARLO — 20 mil rodadas por cenário (FIXO, não recalcula)</t>
+          <t>MONTE CARLO — 200 mil rodadas por cenário (FIXO, não recalcula)</t>
         </is>
       </c>
     </row>
@@ -7748,13 +8304,13 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>0.87515</v>
+        <v>0.87807</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>0.67305</v>
+        <v>0.669355</v>
       </c>
       <c r="D5" s="27" t="n">
-        <v>0.44495</v>
+        <v>0.44232</v>
       </c>
     </row>
     <row r="6">
@@ -7764,13 +8320,13 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>0.0402</v>
+        <v>0.03814</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>0.17445</v>
+        <v>0.17374</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>0.38915</v>
+        <v>0.39148</v>
       </c>
     </row>
     <row r="7">
@@ -7780,13 +8336,13 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.04095</v>
+        <v>0.038695</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.1902</v>
+        <v>0.188425</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.48255</v>
+        <v>0.485415</v>
       </c>
     </row>
     <row r="8">
@@ -7796,13 +8352,13 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>-44674.789625</v>
+        <v>-43876.1013425</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-12007.114125</v>
+        <v>-11403.01613</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>65364.79125</v>
+        <v>63264.648615</v>
       </c>
     </row>
     <row r="9">
@@ -7834,7 +8390,7 @@
         <v>-37870</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>20985</v>
+        <v>24980</v>
       </c>
     </row>
     <row r="11">
@@ -7847,10 +8403,10 @@
         <v>-17820</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>70420</v>
+        <v>69825</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>243330</v>
+        <v>237635</v>
       </c>
     </row>
     <row r="12">
@@ -7860,13 +8416,13 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>1312.801875</v>
+        <v>1249.0314375</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>10655.423625</v>
+        <v>10689.380625</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>50205.42449999999</v>
+        <v>50699.25629999998</v>
       </c>
     </row>
     <row r="13">
@@ -7892,13 +8448,13 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>0.95025</v>
+        <v>0.94006</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>0.72295</v>
+        <v>0.718475</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>0.4342</v>
+        <v>0.43162</v>
       </c>
     </row>
     <row r="17">
@@ -7915,13 +8471,13 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>-44674.789625</v>
+        <v>-43876.1013425</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>-12007.114125</v>
+        <v>-11403.01613</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>65364.79125</v>
+        <v>63264.648615</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
UFC CACE: contrato de projetos R$ 7,2 mi (obra R$ 87 mi) com margem e horas proprias
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpMcBDEADLWoT4jSWTrqdN
</commit_message>
<xml_diff>
--- a/concursos/PROJECAO_CONCURSOS_2026_2028.xlsx
+++ b/concursos/PROJECAO_CONCURSOS_2026_2028.xlsx
@@ -118,6 +118,7 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -125,7 +126,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1723,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -2095,7 +2095,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>UFC CACE — valor da obra</t>
+          <t>UFC CACE — contrato de projetos (arquitetura + complementares)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2114,14 +2114,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Dado seu: R$ 7,2 mi.</t>
+          <t>Dado seu: R$ 7,2 mi. A obra é de R$ 87 mi (só contexto, não entra na conta).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UFC CACE — honorário do projeto como % da obra</t>
+          <t>UFC CACE — margem sobre o contrato (depois de pagar as complementares)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2130,50 +2130,50 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>0.05</v>
+        <v>0.35</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>0.05</v>
+        <v>0.35</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>0.05</v>
+        <v>0.35</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>CHUTE. Projeto completo (arq + complementares) costuma ficar em 4–6% da obra. Confira o edital.</t>
+          <t>CHUTE. Engenharias subcontratadas levam a maior parte; confira o edital e as cotações.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Margem sobre o honorário (depois de equipe/terceiros)</t>
+          <t>UFC CACE — horas SUAS na execução (o resto é equipe)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E19" s="13" t="n">
-        <v>0.55</v>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E19" s="16" t="n">
+        <v>2500</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Chute.</t>
+          <t>CHUTE. Se ganhar, você vai precisar de equipe.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sua parte do contrato (divisão com a JOJO/sócios)</t>
+          <t>Margem sobre o honorário (depois de equipe/terceiros)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2182,24 +2182,24 @@
         </is>
       </c>
       <c r="C20" s="13" t="n">
-        <v>0.7</v>
+        <v>0.55</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>0.7</v>
+        <v>0.55</v>
       </c>
       <c r="E20" s="13" t="n">
-        <v>0.7</v>
+        <v>0.55</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Chute. Na planilha antiga estava 100%, o que superestima.</t>
+          <t>Chute.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Imposto sobre prêmios</t>
+          <t>Sua parte do contrato (divisão com a JOJO/sócios)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2208,24 +2208,24 @@
         </is>
       </c>
       <c r="C21" s="13" t="n">
-        <v>0.15</v>
+        <v>0.7</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.15</v>
+        <v>0.7</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>0.15</v>
+        <v>0.7</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Chute. Confirme com contador.</t>
+          <t>Chute. Na planilha antiga estava 100%, o que superestima.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Imposto sobre contratos</t>
+          <t>Imposto sobre prêmios</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2234,50 +2234,50 @@
         </is>
       </c>
       <c r="C22" s="13" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Chute (Simples/Lucro presumido).</t>
+          <t>Chute. Confirme com contador.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Horas por concurso nacional grande</t>
+          <t>Imposto sobre contratos</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="C23" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D23" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="E23" s="16" t="n">
-        <v>100</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>0.16</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Faixa que dei antes: 60–120 h.</t>
+          <t>Chute (Simples/Lucro presumido).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Horas por concurso internacional</t>
+          <t>Horas por concurso nacional grande</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2285,25 +2285,25 @@
           <t>h</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="D24" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="E24" s="16" t="n">
-        <v>70</v>
+      <c r="C24" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>100</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Estimativa.</t>
+          <t>Faixa que dei antes: 60–120 h.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Horas de execução de um contrato (anteprojeto→executivo)</t>
+          <t>Horas por concurso internacional</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2311,25 +2311,25 @@
           <t>h</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D25" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E25" s="16" t="n">
-        <v>1200</v>
+      <c r="C25" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="D25" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>70</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Chute. Pesa na capacidade em 2028.</t>
+          <t>Estimativa.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Teto de horas por trimestre (concurso + contrato)</t>
+          <t>Horas de execução de um contrato (anteprojeto→executivo)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2337,155 +2337,155 @@
           <t>h</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n">
-        <v>480</v>
-      </c>
-      <c r="D26" s="16" t="n">
-        <v>480</v>
-      </c>
-      <c r="E26" s="16" t="n">
-        <v>480</v>
+      <c r="C26" s="17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>1200</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>160 h/mês, o teto que usei na planilha.</t>
+          <t>Chute. Pesa na capacidade em 2028.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Valor da sua hora (custo de oportunidade)</t>
+          <t>Teto de horas por trimestre (concurso + contrato)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R$/h</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>120</v>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>480</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <v>480</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>480</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>A mesma R$ 120/h da planilha anterior.</t>
+          <t>160 h/mês, o teto que usei na planilha.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ferramentas (Claude, Magnific, licenças)</t>
+          <t>Valor da sua hora (custo de oportunidade)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R$/mês</t>
+          <t>R$/h</t>
         </is>
       </c>
       <c r="C28" s="14" t="n">
-        <v>2500</v>
+        <v>120</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>2500</v>
+        <v>120</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>2500</v>
+        <v>120</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Faixa que dei antes: R$ 1,5–4 mil/mês.</t>
+          <t>A mesma R$ 120/h da planilha anterior.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Parte das ferramentas atribuída aos concursos</t>
+          <t>Ferramentas (Claude, Magnific, licenças)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D29" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E29" s="13" t="n">
-        <v>0.6</v>
+          <t>R$/mês</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>2500</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Chute. O resto serve à perna 2 e a outros trabalhos.</t>
+          <t>Faixa que dei antes: R$ 1,5–4 mil/mês.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inscrição média de concurso internacional</t>
+          <t>Parte das ferramentas atribuída aos concursos</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>R$</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="n">
-        <v>620</v>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>620</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>620</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>0.6</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>≈ € 100 × câmbio.</t>
+          <t>Chute. O resto serve à perna 2 e a outros trabalhos.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CNPJ + contabilidade (a partir de T1/27)</t>
+          <t>Inscrição média de concurso internacional</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>R$/mês</t>
+          <t>R$</t>
         </is>
       </c>
       <c r="C31" s="14" t="n">
-        <v>600</v>
+        <v>620</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>600</v>
+        <v>620</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>600</v>
+        <v>620</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Chute. Assume o CNPJ aberto até dez/2026.</t>
+          <t>≈ € 100 × câmbio.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Renda mensal da 'perna 2' (PSCIP/PICIP, Revit, casa)</t>
+          <t>CNPJ + contabilidade (a partir de T1/27)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2494,50 +2494,50 @@
         </is>
       </c>
       <c r="C32" s="14" t="n">
-        <v>6000</v>
+        <v>600</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>7000</v>
+        <v>600</v>
       </c>
       <c r="E32" s="14" t="n">
-        <v>8000</v>
+        <v>600</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CHUTE TOTAL. Troque pelo seu número real.</t>
+          <t>Chute. Assume o CNPJ aberto até dez/2026.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Crescimento anual da perna 2</t>
+          <t>Renda mensal da 'perna 2' (PSCIP/PICIP, Revit, casa)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E33" s="13" t="n">
-        <v>0.12</v>
+          <t>R$/mês</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>8000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Chute.</t>
+          <t>CHUTE TOTAL. Troque pelo seu número real.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alta da perna 2 após ganhar autoridade (menção/1º)</t>
+          <t>Crescimento anual da perna 2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2549,38 +2549,64 @@
         <v>0</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="E34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.12</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Cliente privado paga mais depois de prêmio. Chute.</t>
+          <t>Chute.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Alta da perna 2 após ganhar autoridade (menção/1º)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E35" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Cliente privado paga mais depois de prêmio. Chute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Trimestre (nº) em que a alta começa (1=T4/26 … 9=T4/28)</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>nº</t>
         </is>
       </c>
-      <c r="C35" s="16" t="n">
+      <c r="C36" s="17" t="n">
         <v>99</v>
       </c>
-      <c r="D35" s="16" t="n">
+      <c r="D36" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="E35" s="16" t="n">
+      <c r="E36" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>99 = nunca acontece.</t>
         </is>
@@ -2629,62 +2655,62 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Unid.</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>T4/26</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>T1/27</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>T2/27</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>T3/27</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>T4/27</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>T1/28</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>T2/28</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>T3/28</t>
         </is>
       </c>
-      <c r="K4" s="17" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>T4/28</t>
         </is>
       </c>
-      <c r="L4" s="17" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2727,22 +2753,22 @@
       <c r="L5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>ENTRADAS</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="21" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="21" t="n"/>
+      <c r="L6" s="21" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2755,31 +2781,31 @@
           <t>nº</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="16" t="n">
         <v>1</v>
       </c>
       <c r="L7" s="22">
@@ -2798,31 +2824,31 @@
           <t>nº</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="16" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="22">
@@ -2831,22 +2857,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>RESULTADOS (saem 1 trimestre após a inscrição)</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="21" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3107,22 +3133,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>CONTRATOS (pagam 3 trimestres após o resultado, em 4 parcelas)</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="20" t="n"/>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="20" t="n"/>
+      <c r="B15" s="20" t="inlineStr"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="21" t="n"/>
+      <c r="L15" s="21" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3188,39 +3214,39 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>C16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((C16-C46)*Premissas!$C$20+C46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>D16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((D16-D46)*Premissas!$C$20+D46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>E16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((E16-E46)*Premissas!$C$20+E46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>F16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((F16-F46)*Premissas!$C$20+F46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>G16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((G16-G46)*Premissas!$C$20+G46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>H16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((H16-H46)*Premissas!$C$20+H46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>I16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((I16-I46)*Premissas!$C$20+I46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="J17" s="8">
-        <f>J16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((J16-J46)*Premissas!$C$20+J46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="K17" s="8">
-        <f>K16*Premissas!$C$19*Premissas!$C$20</f>
+        <f>((K16-K46)*Premissas!$C$20+K46*Premissas!$C$18)*Premissas!$C$21</f>
         <v/>
       </c>
       <c r="L17" s="23">
@@ -3240,39 +3266,39 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>Premissas!$C$25/4*0+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
+        <f>Premissas!$C$26/4*0+Premissas!$C$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="D18" s="7">
-        <f>Premissas!$C$25/4*0+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
+        <f>Premissas!$C$26/4*0+Premissas!$C$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>Premissas!$C$25/4*0+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
+        <f>Premissas!$C$26/4*0+Premissas!$C$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>Premissas!$C$25/4*SUM(C14:C14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
+        <f>Premissas!$C$26/4*SUM(C14:C14)+Premissas!$C$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>Premissas!$C$25/4*SUM(C14:D14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
+        <f>Premissas!$C$26/4*SUM(C14:D14)+Premissas!$C$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>Premissas!$C$25/4*SUM(C14:E14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
+        <f>Premissas!$C$26/4*SUM(C14:E14)+Premissas!$C$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>Premissas!$C$25/4*SUM(C14:F14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
+        <f>Premissas!$C$26/4*SUM(C14:F14)+Premissas!$C$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="J18" s="7">
-        <f>Premissas!$C$25/4*SUM(D14:G14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*1</f>
+        <f>Premissas!$C$26/4*SUM(D14:G14)+Premissas!$C$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>Premissas!$C$25/4*SUM(E14:H14)+Premissas!$C$25*Premissas!$C$17*Premissas!$C$18/Premissas!$C$15/4*$D$45*0</f>
+        <f>Premissas!$C$26/4*SUM(E14:H14)+Premissas!$C$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -3281,22 +3307,22 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>HORAS</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="n"/>
-      <c r="H19" s="20" t="n"/>
-      <c r="I19" s="20" t="n"/>
-      <c r="J19" s="20" t="n"/>
-      <c r="K19" s="20" t="n"/>
-      <c r="L19" s="20" t="n"/>
+      <c r="B19" s="20" t="inlineStr"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="21" t="n"/>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3310,39 +3336,39 @@
         </is>
       </c>
       <c r="C20" s="7">
-        <f>C7*Premissas!$C$23+C8*Premissas!$C$24</f>
+        <f>C7*Premissas!$C$24+C8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="D20" s="7">
-        <f>D7*Premissas!$C$23+D8*Premissas!$C$24</f>
+        <f>D7*Premissas!$C$24+D8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>E7*Premissas!$C$23+E8*Premissas!$C$24</f>
+        <f>E7*Premissas!$C$24+E8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>F7*Premissas!$C$23+F8*Premissas!$C$24</f>
+        <f>F7*Premissas!$C$24+F8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>G7*Premissas!$C$23+G8*Premissas!$C$24</f>
+        <f>G7*Premissas!$C$24+G8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>H7*Premissas!$C$23+H8*Premissas!$C$24</f>
+        <f>H7*Premissas!$C$24+H8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>I7*Premissas!$C$23+I8*Premissas!$C$24</f>
+        <f>I7*Premissas!$C$24+I8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="J20" s="7">
-        <f>J7*Premissas!$C$23+J8*Premissas!$C$24</f>
+        <f>J7*Premissas!$C$24+J8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>K7*Premissas!$C$23+K8*Premissas!$C$24</f>
+        <f>K7*Premissas!$C$24+K8*Premissas!$C$25</f>
         <v/>
       </c>
       <c r="L20" s="22">
@@ -3411,39 +3437,39 @@
         </is>
       </c>
       <c r="C22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="D22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="J22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>Premissas!$C$26</f>
+        <f>Premissas!$C$27</f>
         <v/>
       </c>
       <c r="L22" s="7" t="n"/>
@@ -3494,22 +3520,22 @@
       <c r="L23" s="25" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>CAIXA DOS CONCURSOS</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr"/>
-      <c r="C24" s="20" t="n"/>
-      <c r="D24" s="20" t="n"/>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="n"/>
-      <c r="H24" s="20" t="n"/>
-      <c r="I24" s="20" t="n"/>
-      <c r="J24" s="20" t="n"/>
-      <c r="K24" s="20" t="n"/>
-      <c r="L24" s="20" t="n"/>
+      <c r="B24" s="20" t="inlineStr"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="21" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="21" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3627,39 +3653,39 @@
         </is>
       </c>
       <c r="C27" s="8">
-        <f>-(C25*Premissas!$C$21+C26*Premissas!$C$22)</f>
+        <f>-(C25*Premissas!$C$22+C26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>-(D25*Premissas!$C$21+D26*Premissas!$C$22)</f>
+        <f>-(D25*Premissas!$C$22+D26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>-(E25*Premissas!$C$21+E26*Premissas!$C$22)</f>
+        <f>-(E25*Premissas!$C$22+E26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>-(F25*Premissas!$C$21+F26*Premissas!$C$22)</f>
+        <f>-(F25*Premissas!$C$22+F26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="G27" s="8">
-        <f>-(G25*Premissas!$C$21+G26*Premissas!$C$22)</f>
+        <f>-(G25*Premissas!$C$22+G26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="H27" s="8">
-        <f>-(H25*Premissas!$C$21+H26*Premissas!$C$22)</f>
+        <f>-(H25*Premissas!$C$22+H26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="I27" s="8">
-        <f>-(I25*Premissas!$C$21+I26*Premissas!$C$22)</f>
+        <f>-(I25*Premissas!$C$22+I26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>-(J25*Premissas!$C$21+J26*Premissas!$C$22)</f>
+        <f>-(J25*Premissas!$C$22+J26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="K27" s="8">
-        <f>-(K25*Premissas!$C$21+K26*Premissas!$C$22)</f>
+        <f>-(K25*Premissas!$C$22+K26*Premissas!$C$23)</f>
         <v/>
       </c>
       <c r="L27" s="23">
@@ -3679,39 +3705,39 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="G28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="H28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="I28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="J28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="K28" s="8">
-        <f>-3*Premissas!$C$28*Premissas!$C$29</f>
+        <f>-3*Premissas!$C$29*Premissas!$C$30</f>
         <v/>
       </c>
       <c r="L28" s="23">
@@ -3731,39 +3757,39 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>-C8*Premissas!$C$30</f>
+        <f>-C8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>-D8*Premissas!$C$30</f>
+        <f>-D8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>-E8*Premissas!$C$30</f>
+        <f>-E8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>-F8*Premissas!$C$30</f>
+        <f>-F8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>-G8*Premissas!$C$30</f>
+        <f>-G8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>-H8*Premissas!$C$30</f>
+        <f>-H8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>-I8*Premissas!$C$30</f>
+        <f>-I8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>-J8*Premissas!$C$30</f>
+        <f>-J8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>-K8*Premissas!$C$30</f>
+        <f>-K8*Premissas!$C$31</f>
         <v/>
       </c>
       <c r="L29" s="23">
@@ -3786,35 +3812,35 @@
         <v>0</v>
       </c>
       <c r="D30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="G30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="H30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="I30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="J30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="K30" s="8">
-        <f>-3*Premissas!$C$31</f>
+        <f>-3*Premissas!$C$32</f>
         <v/>
       </c>
       <c r="L30" s="23">
@@ -3886,39 +3912,39 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>-C20*Premissas!$C$27</f>
+        <f>-C20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="D32" s="8">
-        <f>-D20*Premissas!$C$27</f>
+        <f>-D20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="E32" s="8">
-        <f>-E20*Premissas!$C$27</f>
+        <f>-E20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="F32" s="8">
-        <f>-F20*Premissas!$C$27</f>
+        <f>-F20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="G32" s="8">
-        <f>-G20*Premissas!$C$27</f>
+        <f>-G20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="H32" s="8">
-        <f>-H20*Premissas!$C$27</f>
+        <f>-H20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="I32" s="8">
-        <f>-I20*Premissas!$C$27</f>
+        <f>-I20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="J32" s="8">
-        <f>-J20*Premissas!$C$27</f>
+        <f>-J20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="K32" s="8">
-        <f>-K20*Premissas!$C$27</f>
+        <f>-K20*Premissas!$C$28</f>
         <v/>
       </c>
       <c r="L32" s="23">
@@ -3979,22 +4005,22 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>RENDA TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="19" t="inlineStr"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="n"/>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="n"/>
-      <c r="H34" s="20" t="n"/>
-      <c r="I34" s="20" t="n"/>
-      <c r="J34" s="20" t="n"/>
-      <c r="K34" s="20" t="n"/>
-      <c r="L34" s="20" t="n"/>
+      <c r="B34" s="20" t="inlineStr"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="21" t="n"/>
+      <c r="I34" s="21" t="n"/>
+      <c r="J34" s="21" t="n"/>
+      <c r="K34" s="21" t="n"/>
+      <c r="L34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4008,39 +4034,39 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="H35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="I35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="J35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="K35" s="8">
-        <f>3*Premissas!$C$32*(1+Premissas!$C$33)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$C$35,Premissas!$C$34,0))</f>
+        <f>3*Premissas!$C$33*(1+Premissas!$C$34)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$C$36,Premissas!$C$35,0))</f>
         <v/>
       </c>
       <c r="L35" s="23">
@@ -4251,22 +4277,22 @@
       <c r="L39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>CARTEIRA</t>
         </is>
       </c>
-      <c r="B40" s="19" t="inlineStr"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="20" t="n"/>
-      <c r="F40" s="20" t="n"/>
-      <c r="G40" s="20" t="n"/>
-      <c r="H40" s="20" t="n"/>
-      <c r="I40" s="20" t="n"/>
-      <c r="J40" s="20" t="n"/>
-      <c r="K40" s="20" t="n"/>
-      <c r="L40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr"/>
+      <c r="C40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="21" t="n"/>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="21" t="n"/>
+      <c r="H40" s="21" t="n"/>
+      <c r="I40" s="21" t="n"/>
+      <c r="J40" s="21" t="n"/>
+      <c r="K40" s="21" t="n"/>
+      <c r="L40" s="21" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4314,27 +4340,27 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="23">
-        <f>(L14*Premissas!$C$15+L45*Premissas!$C$17*Premissas!$C$18)*Premissas!$C$19*Premissas!$C$20*(1-Premissas!$C$22)-L26*(1-Premissas!$C$22)</f>
+        <f>(L14*Premissas!$C$15*Premissas!$C$20+L45*Premissas!$C$17*Premissas!$C$18)*Premissas!$C$21*(1-Premissas!$C$23)-L26*(1-Premissas!$C$23)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>UFC CACE (entrega 21/10/2026, resultado em T1/27) — separado do genérico</t>
         </is>
       </c>
-      <c r="B43" s="19" t="inlineStr"/>
-      <c r="C43" s="20" t="n"/>
-      <c r="D43" s="20" t="n"/>
-      <c r="E43" s="20" t="n"/>
-      <c r="F43" s="20" t="n"/>
-      <c r="G43" s="20" t="n"/>
-      <c r="H43" s="20" t="n"/>
-      <c r="I43" s="20" t="n"/>
-      <c r="J43" s="20" t="n"/>
-      <c r="K43" s="20" t="n"/>
-      <c r="L43" s="20" t="n"/>
+      <c r="B43" s="20" t="inlineStr"/>
+      <c r="C43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="21" t="n"/>
+      <c r="F43" s="21" t="n"/>
+      <c r="G43" s="21" t="n"/>
+      <c r="H43" s="21" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="21" t="n"/>
+      <c r="K43" s="21" t="n"/>
+      <c r="L43" s="21" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4448,19 +4474,19 @@
         <v>0</v>
       </c>
       <c r="G46" s="8">
-        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <f>Premissas!$C$17/4*$D$45</f>
         <v/>
       </c>
       <c r="H46" s="8">
-        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <f>Premissas!$C$17/4*$D$45</f>
         <v/>
       </c>
       <c r="I46" s="8">
-        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <f>Premissas!$C$17/4*$D$45</f>
         <v/>
       </c>
       <c r="J46" s="8">
-        <f>Premissas!$C$17*Premissas!$C$18/4*$D$45</f>
+        <f>Premissas!$C$17/4*$D$45</f>
         <v/>
       </c>
       <c r="K46" s="8" t="n">
@@ -4514,62 +4540,62 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Unid.</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>T4/26</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>T1/27</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>T2/27</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>T3/27</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>T4/27</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>T1/28</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>T2/28</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>T3/28</t>
         </is>
       </c>
-      <c r="K4" s="17" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>T4/28</t>
         </is>
       </c>
-      <c r="L4" s="17" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4612,22 +4638,22 @@
       <c r="L5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>ENTRADAS</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="21" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="21" t="n"/>
+      <c r="L6" s="21" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4640,31 +4666,31 @@
           <t>nº</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L7" s="22">
@@ -4683,31 +4709,31 @@
           <t>nº</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="16" t="n">
         <v>1</v>
       </c>
       <c r="L8" s="22">
@@ -4716,22 +4742,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>RESULTADOS (saem 1 trimestre após a inscrição)</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="21" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4992,22 +5018,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>CONTRATOS (pagam 3 trimestres após o resultado, em 4 parcelas)</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="20" t="n"/>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="20" t="n"/>
+      <c r="B15" s="20" t="inlineStr"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="21" t="n"/>
+      <c r="L15" s="21" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5073,39 +5099,39 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>C16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((C16-C46)*Premissas!$D$20+C46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>D16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((D16-D46)*Premissas!$D$20+D46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>E16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((E16-E46)*Premissas!$D$20+E46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>F16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((F16-F46)*Premissas!$D$20+F46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>G16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((G16-G46)*Premissas!$D$20+G46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>H16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((H16-H46)*Premissas!$D$20+H46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>I16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((I16-I46)*Premissas!$D$20+I46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="J17" s="8">
-        <f>J16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((J16-J46)*Premissas!$D$20+J46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="K17" s="8">
-        <f>K16*Premissas!$D$19*Premissas!$D$20</f>
+        <f>((K16-K46)*Premissas!$D$20+K46*Premissas!$D$18)*Premissas!$D$21</f>
         <v/>
       </c>
       <c r="L17" s="23">
@@ -5125,39 +5151,39 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>Premissas!$D$25/4*0+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
+        <f>Premissas!$D$26/4*0+Premissas!$D$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="D18" s="7">
-        <f>Premissas!$D$25/4*0+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
+        <f>Premissas!$D$26/4*0+Premissas!$D$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>Premissas!$D$25/4*0+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
+        <f>Premissas!$D$26/4*0+Premissas!$D$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>Premissas!$D$25/4*SUM(C14:C14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
+        <f>Premissas!$D$26/4*SUM(C14:C14)+Premissas!$D$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>Premissas!$D$25/4*SUM(C14:D14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
+        <f>Premissas!$D$26/4*SUM(C14:D14)+Premissas!$D$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>Premissas!$D$25/4*SUM(C14:E14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
+        <f>Premissas!$D$26/4*SUM(C14:E14)+Premissas!$D$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>Premissas!$D$25/4*SUM(C14:F14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
+        <f>Premissas!$D$26/4*SUM(C14:F14)+Premissas!$D$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="J18" s="7">
-        <f>Premissas!$D$25/4*SUM(D14:G14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*1</f>
+        <f>Premissas!$D$26/4*SUM(D14:G14)+Premissas!$D$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>Premissas!$D$25/4*SUM(E14:H14)+Premissas!$D$25*Premissas!$D$17*Premissas!$D$18/Premissas!$D$15/4*$D$45*0</f>
+        <f>Premissas!$D$26/4*SUM(E14:H14)+Premissas!$D$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -5166,22 +5192,22 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>HORAS</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="n"/>
-      <c r="H19" s="20" t="n"/>
-      <c r="I19" s="20" t="n"/>
-      <c r="J19" s="20" t="n"/>
-      <c r="K19" s="20" t="n"/>
-      <c r="L19" s="20" t="n"/>
+      <c r="B19" s="20" t="inlineStr"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="21" t="n"/>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5195,39 +5221,39 @@
         </is>
       </c>
       <c r="C20" s="7">
-        <f>C7*Premissas!$D$23+C8*Premissas!$D$24</f>
+        <f>C7*Premissas!$D$24+C8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="D20" s="7">
-        <f>D7*Premissas!$D$23+D8*Premissas!$D$24</f>
+        <f>D7*Premissas!$D$24+D8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>E7*Premissas!$D$23+E8*Premissas!$D$24</f>
+        <f>E7*Premissas!$D$24+E8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>F7*Premissas!$D$23+F8*Premissas!$D$24</f>
+        <f>F7*Premissas!$D$24+F8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>G7*Premissas!$D$23+G8*Premissas!$D$24</f>
+        <f>G7*Premissas!$D$24+G8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>H7*Premissas!$D$23+H8*Premissas!$D$24</f>
+        <f>H7*Premissas!$D$24+H8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>I7*Premissas!$D$23+I8*Premissas!$D$24</f>
+        <f>I7*Premissas!$D$24+I8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="J20" s="7">
-        <f>J7*Premissas!$D$23+J8*Premissas!$D$24</f>
+        <f>J7*Premissas!$D$24+J8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>K7*Premissas!$D$23+K8*Premissas!$D$24</f>
+        <f>K7*Premissas!$D$24+K8*Premissas!$D$25</f>
         <v/>
       </c>
       <c r="L20" s="22">
@@ -5296,39 +5322,39 @@
         </is>
       </c>
       <c r="C22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="D22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="J22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>Premissas!$D$26</f>
+        <f>Premissas!$D$27</f>
         <v/>
       </c>
       <c r="L22" s="7" t="n"/>
@@ -5379,22 +5405,22 @@
       <c r="L23" s="25" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>CAIXA DOS CONCURSOS</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr"/>
-      <c r="C24" s="20" t="n"/>
-      <c r="D24" s="20" t="n"/>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="n"/>
-      <c r="H24" s="20" t="n"/>
-      <c r="I24" s="20" t="n"/>
-      <c r="J24" s="20" t="n"/>
-      <c r="K24" s="20" t="n"/>
-      <c r="L24" s="20" t="n"/>
+      <c r="B24" s="20" t="inlineStr"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="21" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="21" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5512,39 +5538,39 @@
         </is>
       </c>
       <c r="C27" s="8">
-        <f>-(C25*Premissas!$D$21+C26*Premissas!$D$22)</f>
+        <f>-(C25*Premissas!$D$22+C26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>-(D25*Premissas!$D$21+D26*Premissas!$D$22)</f>
+        <f>-(D25*Premissas!$D$22+D26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>-(E25*Premissas!$D$21+E26*Premissas!$D$22)</f>
+        <f>-(E25*Premissas!$D$22+E26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>-(F25*Premissas!$D$21+F26*Premissas!$D$22)</f>
+        <f>-(F25*Premissas!$D$22+F26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="G27" s="8">
-        <f>-(G25*Premissas!$D$21+G26*Premissas!$D$22)</f>
+        <f>-(G25*Premissas!$D$22+G26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="H27" s="8">
-        <f>-(H25*Premissas!$D$21+H26*Premissas!$D$22)</f>
+        <f>-(H25*Premissas!$D$22+H26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="I27" s="8">
-        <f>-(I25*Premissas!$D$21+I26*Premissas!$D$22)</f>
+        <f>-(I25*Premissas!$D$22+I26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>-(J25*Premissas!$D$21+J26*Premissas!$D$22)</f>
+        <f>-(J25*Premissas!$D$22+J26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="K27" s="8">
-        <f>-(K25*Premissas!$D$21+K26*Premissas!$D$22)</f>
+        <f>-(K25*Premissas!$D$22+K26*Premissas!$D$23)</f>
         <v/>
       </c>
       <c r="L27" s="23">
@@ -5564,39 +5590,39 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="G28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="H28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="I28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="J28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="K28" s="8">
-        <f>-3*Premissas!$D$28*Premissas!$D$29</f>
+        <f>-3*Premissas!$D$29*Premissas!$D$30</f>
         <v/>
       </c>
       <c r="L28" s="23">
@@ -5616,39 +5642,39 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>-C8*Premissas!$D$30</f>
+        <f>-C8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>-D8*Premissas!$D$30</f>
+        <f>-D8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>-E8*Premissas!$D$30</f>
+        <f>-E8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>-F8*Premissas!$D$30</f>
+        <f>-F8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>-G8*Premissas!$D$30</f>
+        <f>-G8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>-H8*Premissas!$D$30</f>
+        <f>-H8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>-I8*Premissas!$D$30</f>
+        <f>-I8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>-J8*Premissas!$D$30</f>
+        <f>-J8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>-K8*Premissas!$D$30</f>
+        <f>-K8*Premissas!$D$31</f>
         <v/>
       </c>
       <c r="L29" s="23">
@@ -5671,35 +5697,35 @@
         <v>0</v>
       </c>
       <c r="D30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="G30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="H30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="I30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="J30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="K30" s="8">
-        <f>-3*Premissas!$D$31</f>
+        <f>-3*Premissas!$D$32</f>
         <v/>
       </c>
       <c r="L30" s="23">
@@ -5771,39 +5797,39 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>-C20*Premissas!$D$27</f>
+        <f>-C20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="D32" s="8">
-        <f>-D20*Premissas!$D$27</f>
+        <f>-D20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="E32" s="8">
-        <f>-E20*Premissas!$D$27</f>
+        <f>-E20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="F32" s="8">
-        <f>-F20*Premissas!$D$27</f>
+        <f>-F20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="G32" s="8">
-        <f>-G20*Premissas!$D$27</f>
+        <f>-G20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="H32" s="8">
-        <f>-H20*Premissas!$D$27</f>
+        <f>-H20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="I32" s="8">
-        <f>-I20*Premissas!$D$27</f>
+        <f>-I20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="J32" s="8">
-        <f>-J20*Premissas!$D$27</f>
+        <f>-J20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="K32" s="8">
-        <f>-K20*Premissas!$D$27</f>
+        <f>-K20*Premissas!$D$28</f>
         <v/>
       </c>
       <c r="L32" s="23">
@@ -5864,22 +5890,22 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>RENDA TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="19" t="inlineStr"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="n"/>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="n"/>
-      <c r="H34" s="20" t="n"/>
-      <c r="I34" s="20" t="n"/>
-      <c r="J34" s="20" t="n"/>
-      <c r="K34" s="20" t="n"/>
-      <c r="L34" s="20" t="n"/>
+      <c r="B34" s="20" t="inlineStr"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="21" t="n"/>
+      <c r="I34" s="21" t="n"/>
+      <c r="J34" s="21" t="n"/>
+      <c r="K34" s="21" t="n"/>
+      <c r="L34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5893,39 +5919,39 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="H35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="I35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="J35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="K35" s="8">
-        <f>3*Premissas!$D$32*(1+Premissas!$D$33)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$D$35,Premissas!$D$34,0))</f>
+        <f>3*Premissas!$D$33*(1+Premissas!$D$34)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$D$36,Premissas!$D$35,0))</f>
         <v/>
       </c>
       <c r="L35" s="23">
@@ -6136,22 +6162,22 @@
       <c r="L39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>CARTEIRA</t>
         </is>
       </c>
-      <c r="B40" s="19" t="inlineStr"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="20" t="n"/>
-      <c r="F40" s="20" t="n"/>
-      <c r="G40" s="20" t="n"/>
-      <c r="H40" s="20" t="n"/>
-      <c r="I40" s="20" t="n"/>
-      <c r="J40" s="20" t="n"/>
-      <c r="K40" s="20" t="n"/>
-      <c r="L40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr"/>
+      <c r="C40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="21" t="n"/>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="21" t="n"/>
+      <c r="H40" s="21" t="n"/>
+      <c r="I40" s="21" t="n"/>
+      <c r="J40" s="21" t="n"/>
+      <c r="K40" s="21" t="n"/>
+      <c r="L40" s="21" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6199,27 +6225,27 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="23">
-        <f>(L14*Premissas!$D$15+L45*Premissas!$D$17*Premissas!$D$18)*Premissas!$D$19*Premissas!$D$20*(1-Premissas!$D$22)-L26*(1-Premissas!$D$22)</f>
+        <f>(L14*Premissas!$D$15*Premissas!$D$20+L45*Premissas!$D$17*Premissas!$D$18)*Premissas!$D$21*(1-Premissas!$D$23)-L26*(1-Premissas!$D$23)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>UFC CACE (entrega 21/10/2026, resultado em T1/27) — separado do genérico</t>
         </is>
       </c>
-      <c r="B43" s="19" t="inlineStr"/>
-      <c r="C43" s="20" t="n"/>
-      <c r="D43" s="20" t="n"/>
-      <c r="E43" s="20" t="n"/>
-      <c r="F43" s="20" t="n"/>
-      <c r="G43" s="20" t="n"/>
-      <c r="H43" s="20" t="n"/>
-      <c r="I43" s="20" t="n"/>
-      <c r="J43" s="20" t="n"/>
-      <c r="K43" s="20" t="n"/>
-      <c r="L43" s="20" t="n"/>
+      <c r="B43" s="20" t="inlineStr"/>
+      <c r="C43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="21" t="n"/>
+      <c r="F43" s="21" t="n"/>
+      <c r="G43" s="21" t="n"/>
+      <c r="H43" s="21" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="21" t="n"/>
+      <c r="K43" s="21" t="n"/>
+      <c r="L43" s="21" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6333,19 +6359,19 @@
         <v>0</v>
       </c>
       <c r="G46" s="8">
-        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <f>Premissas!$D$17/4*$D$45</f>
         <v/>
       </c>
       <c r="H46" s="8">
-        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <f>Premissas!$D$17/4*$D$45</f>
         <v/>
       </c>
       <c r="I46" s="8">
-        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <f>Premissas!$D$17/4*$D$45</f>
         <v/>
       </c>
       <c r="J46" s="8">
-        <f>Premissas!$D$17*Premissas!$D$18/4*$D$45</f>
+        <f>Premissas!$D$17/4*$D$45</f>
         <v/>
       </c>
       <c r="K46" s="8" t="n">
@@ -6399,62 +6425,62 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Unid.</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>T4/26</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>T1/27</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>T2/27</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>T3/27</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>T4/27</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>T1/28</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>T2/28</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>T3/28</t>
         </is>
       </c>
-      <c r="K4" s="17" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>T4/28</t>
         </is>
       </c>
-      <c r="L4" s="17" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -6497,22 +6523,22 @@
       <c r="L5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>ENTRADAS</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="21" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="21" t="n"/>
+      <c r="L6" s="21" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6525,31 +6551,31 @@
           <t>nº</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="16" t="n">
         <v>1</v>
       </c>
       <c r="L7" s="22">
@@ -6568,31 +6594,31 @@
           <t>nº</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="16" t="n">
         <v>1</v>
       </c>
       <c r="L8" s="22">
@@ -6601,22 +6627,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>RESULTADOS (saem 1 trimestre após a inscrição)</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="21" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6877,22 +6903,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>CONTRATOS (pagam 3 trimestres após o resultado, em 4 parcelas)</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="20" t="n"/>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="20" t="n"/>
+      <c r="B15" s="20" t="inlineStr"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="21" t="n"/>
+      <c r="L15" s="21" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6958,39 +6984,39 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>C16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((C16-C46)*Premissas!$E$20+C46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>D16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((D16-D46)*Premissas!$E$20+D46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>E16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((E16-E46)*Premissas!$E$20+E46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>F16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((F16-F46)*Premissas!$E$20+F46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>G16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((G16-G46)*Premissas!$E$20+G46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="H17" s="8">
-        <f>H16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((H16-H46)*Premissas!$E$20+H46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="I17" s="8">
-        <f>I16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((I16-I46)*Premissas!$E$20+I46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="J17" s="8">
-        <f>J16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((J16-J46)*Premissas!$E$20+J46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="K17" s="8">
-        <f>K16*Premissas!$E$19*Premissas!$E$20</f>
+        <f>((K16-K46)*Premissas!$E$20+K46*Premissas!$E$18)*Premissas!$E$21</f>
         <v/>
       </c>
       <c r="L17" s="23">
@@ -7010,39 +7036,39 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>Premissas!$E$25/4*0+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
+        <f>Premissas!$E$26/4*0+Premissas!$E$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="D18" s="7">
-        <f>Premissas!$E$25/4*0+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
+        <f>Premissas!$E$26/4*0+Premissas!$E$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>Premissas!$E$25/4*0+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
+        <f>Premissas!$E$26/4*0+Premissas!$E$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>Premissas!$E$25/4*SUM(C14:C14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
+        <f>Premissas!$E$26/4*SUM(C14:C14)+Premissas!$E$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>Premissas!$E$25/4*SUM(C14:D14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
+        <f>Premissas!$E$26/4*SUM(C14:D14)+Premissas!$E$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>Premissas!$E$25/4*SUM(C14:E14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
+        <f>Premissas!$E$26/4*SUM(C14:E14)+Premissas!$E$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>Premissas!$E$25/4*SUM(C14:F14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
+        <f>Premissas!$E$26/4*SUM(C14:F14)+Premissas!$E$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="J18" s="7">
-        <f>Premissas!$E$25/4*SUM(D14:G14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*1</f>
+        <f>Premissas!$E$26/4*SUM(D14:G14)+Premissas!$E$19/4*$D$45*1</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>Premissas!$E$25/4*SUM(E14:H14)+Premissas!$E$25*Premissas!$E$17*Premissas!$E$18/Premissas!$E$15/4*$D$45*0</f>
+        <f>Premissas!$E$26/4*SUM(E14:H14)+Premissas!$E$19/4*$D$45*0</f>
         <v/>
       </c>
       <c r="L18" s="22">
@@ -7051,22 +7077,22 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>HORAS</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="n"/>
-      <c r="H19" s="20" t="n"/>
-      <c r="I19" s="20" t="n"/>
-      <c r="J19" s="20" t="n"/>
-      <c r="K19" s="20" t="n"/>
-      <c r="L19" s="20" t="n"/>
+      <c r="B19" s="20" t="inlineStr"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="21" t="n"/>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7080,39 +7106,39 @@
         </is>
       </c>
       <c r="C20" s="7">
-        <f>C7*Premissas!$E$23+C8*Premissas!$E$24</f>
+        <f>C7*Premissas!$E$24+C8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="D20" s="7">
-        <f>D7*Premissas!$E$23+D8*Premissas!$E$24</f>
+        <f>D7*Premissas!$E$24+D8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>E7*Premissas!$E$23+E8*Premissas!$E$24</f>
+        <f>E7*Premissas!$E$24+E8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>F7*Premissas!$E$23+F8*Premissas!$E$24</f>
+        <f>F7*Premissas!$E$24+F8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>G7*Premissas!$E$23+G8*Premissas!$E$24</f>
+        <f>G7*Premissas!$E$24+G8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>H7*Premissas!$E$23+H8*Premissas!$E$24</f>
+        <f>H7*Premissas!$E$24+H8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>I7*Premissas!$E$23+I8*Premissas!$E$24</f>
+        <f>I7*Premissas!$E$24+I8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="J20" s="7">
-        <f>J7*Premissas!$E$23+J8*Premissas!$E$24</f>
+        <f>J7*Premissas!$E$24+J8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>K7*Premissas!$E$23+K8*Premissas!$E$24</f>
+        <f>K7*Premissas!$E$24+K8*Premissas!$E$25</f>
         <v/>
       </c>
       <c r="L20" s="22">
@@ -7181,39 +7207,39 @@
         </is>
       </c>
       <c r="C22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="D22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="J22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>Premissas!$E$26</f>
+        <f>Premissas!$E$27</f>
         <v/>
       </c>
       <c r="L22" s="7" t="n"/>
@@ -7264,22 +7290,22 @@
       <c r="L23" s="25" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>CAIXA DOS CONCURSOS</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr"/>
-      <c r="C24" s="20" t="n"/>
-      <c r="D24" s="20" t="n"/>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="n"/>
-      <c r="H24" s="20" t="n"/>
-      <c r="I24" s="20" t="n"/>
-      <c r="J24" s="20" t="n"/>
-      <c r="K24" s="20" t="n"/>
-      <c r="L24" s="20" t="n"/>
+      <c r="B24" s="20" t="inlineStr"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="21" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="21" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7397,39 +7423,39 @@
         </is>
       </c>
       <c r="C27" s="8">
-        <f>-(C25*Premissas!$E$21+C26*Premissas!$E$22)</f>
+        <f>-(C25*Premissas!$E$22+C26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>-(D25*Premissas!$E$21+D26*Premissas!$E$22)</f>
+        <f>-(D25*Premissas!$E$22+D26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>-(E25*Premissas!$E$21+E26*Premissas!$E$22)</f>
+        <f>-(E25*Premissas!$E$22+E26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>-(F25*Premissas!$E$21+F26*Premissas!$E$22)</f>
+        <f>-(F25*Premissas!$E$22+F26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="G27" s="8">
-        <f>-(G25*Premissas!$E$21+G26*Premissas!$E$22)</f>
+        <f>-(G25*Premissas!$E$22+G26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="H27" s="8">
-        <f>-(H25*Premissas!$E$21+H26*Premissas!$E$22)</f>
+        <f>-(H25*Premissas!$E$22+H26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="I27" s="8">
-        <f>-(I25*Premissas!$E$21+I26*Premissas!$E$22)</f>
+        <f>-(I25*Premissas!$E$22+I26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>-(J25*Premissas!$E$21+J26*Premissas!$E$22)</f>
+        <f>-(J25*Premissas!$E$22+J26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="K27" s="8">
-        <f>-(K25*Premissas!$E$21+K26*Premissas!$E$22)</f>
+        <f>-(K25*Premissas!$E$22+K26*Premissas!$E$23)</f>
         <v/>
       </c>
       <c r="L27" s="23">
@@ -7449,39 +7475,39 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="G28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="H28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="I28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="J28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="K28" s="8">
-        <f>-3*Premissas!$E$28*Premissas!$E$29</f>
+        <f>-3*Premissas!$E$29*Premissas!$E$30</f>
         <v/>
       </c>
       <c r="L28" s="23">
@@ -7501,39 +7527,39 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>-C8*Premissas!$E$30</f>
+        <f>-C8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>-D8*Premissas!$E$30</f>
+        <f>-D8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>-E8*Premissas!$E$30</f>
+        <f>-E8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>-F8*Premissas!$E$30</f>
+        <f>-F8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>-G8*Premissas!$E$30</f>
+        <f>-G8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>-H8*Premissas!$E$30</f>
+        <f>-H8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>-I8*Premissas!$E$30</f>
+        <f>-I8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>-J8*Premissas!$E$30</f>
+        <f>-J8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>-K8*Premissas!$E$30</f>
+        <f>-K8*Premissas!$E$31</f>
         <v/>
       </c>
       <c r="L29" s="23">
@@ -7556,35 +7582,35 @@
         <v>0</v>
       </c>
       <c r="D30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="G30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="H30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="I30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="J30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="K30" s="8">
-        <f>-3*Premissas!$E$31</f>
+        <f>-3*Premissas!$E$32</f>
         <v/>
       </c>
       <c r="L30" s="23">
@@ -7656,39 +7682,39 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>-C20*Premissas!$E$27</f>
+        <f>-C20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="D32" s="8">
-        <f>-D20*Premissas!$E$27</f>
+        <f>-D20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="E32" s="8">
-        <f>-E20*Premissas!$E$27</f>
+        <f>-E20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="F32" s="8">
-        <f>-F20*Premissas!$E$27</f>
+        <f>-F20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="G32" s="8">
-        <f>-G20*Premissas!$E$27</f>
+        <f>-G20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="H32" s="8">
-        <f>-H20*Premissas!$E$27</f>
+        <f>-H20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="I32" s="8">
-        <f>-I20*Premissas!$E$27</f>
+        <f>-I20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="J32" s="8">
-        <f>-J20*Premissas!$E$27</f>
+        <f>-J20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="K32" s="8">
-        <f>-K20*Premissas!$E$27</f>
+        <f>-K20*Premissas!$E$28</f>
         <v/>
       </c>
       <c r="L32" s="23">
@@ -7749,22 +7775,22 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>RENDA TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="19" t="inlineStr"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="n"/>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="n"/>
-      <c r="H34" s="20" t="n"/>
-      <c r="I34" s="20" t="n"/>
-      <c r="J34" s="20" t="n"/>
-      <c r="K34" s="20" t="n"/>
-      <c r="L34" s="20" t="n"/>
+      <c r="B34" s="20" t="inlineStr"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="21" t="n"/>
+      <c r="I34" s="21" t="n"/>
+      <c r="J34" s="21" t="n"/>
+      <c r="K34" s="21" t="n"/>
+      <c r="L34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7778,39 +7804,39 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((C5-1)/4)*(1+IF(C5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((D5-1)/4)*(1+IF(D5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((E5-1)/4)*(1+IF(E5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((F5-1)/4)*(1+IF(F5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((G5-1)/4)*(1+IF(G5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="H35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((H5-1)/4)*(1+IF(H5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="I35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((I5-1)/4)*(1+IF(I5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="J35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((J5-1)/4)*(1+IF(J5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="K35" s="8">
-        <f>3*Premissas!$E$32*(1+Premissas!$E$33)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$E$35,Premissas!$E$34,0))</f>
+        <f>3*Premissas!$E$33*(1+Premissas!$E$34)^((K5-1)/4)*(1+IF(K5&gt;=Premissas!$E$36,Premissas!$E$35,0))</f>
         <v/>
       </c>
       <c r="L35" s="23">
@@ -8021,22 +8047,22 @@
       <c r="L39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>CARTEIRA</t>
         </is>
       </c>
-      <c r="B40" s="19" t="inlineStr"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="20" t="n"/>
-      <c r="F40" s="20" t="n"/>
-      <c r="G40" s="20" t="n"/>
-      <c r="H40" s="20" t="n"/>
-      <c r="I40" s="20" t="n"/>
-      <c r="J40" s="20" t="n"/>
-      <c r="K40" s="20" t="n"/>
-      <c r="L40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr"/>
+      <c r="C40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="21" t="n"/>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="21" t="n"/>
+      <c r="H40" s="21" t="n"/>
+      <c r="I40" s="21" t="n"/>
+      <c r="J40" s="21" t="n"/>
+      <c r="K40" s="21" t="n"/>
+      <c r="L40" s="21" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8084,27 +8110,27 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="23">
-        <f>(L14*Premissas!$E$15+L45*Premissas!$E$17*Premissas!$E$18)*Premissas!$E$19*Premissas!$E$20*(1-Premissas!$E$22)-L26*(1-Premissas!$E$22)</f>
+        <f>(L14*Premissas!$E$15*Premissas!$E$20+L45*Premissas!$E$17*Premissas!$E$18)*Premissas!$E$21*(1-Premissas!$E$23)-L26*(1-Premissas!$E$23)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>UFC CACE (entrega 21/10/2026, resultado em T1/27) — separado do genérico</t>
         </is>
       </c>
-      <c r="B43" s="19" t="inlineStr"/>
-      <c r="C43" s="20" t="n"/>
-      <c r="D43" s="20" t="n"/>
-      <c r="E43" s="20" t="n"/>
-      <c r="F43" s="20" t="n"/>
-      <c r="G43" s="20" t="n"/>
-      <c r="H43" s="20" t="n"/>
-      <c r="I43" s="20" t="n"/>
-      <c r="J43" s="20" t="n"/>
-      <c r="K43" s="20" t="n"/>
-      <c r="L43" s="20" t="n"/>
+      <c r="B43" s="20" t="inlineStr"/>
+      <c r="C43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="21" t="n"/>
+      <c r="F43" s="21" t="n"/>
+      <c r="G43" s="21" t="n"/>
+      <c r="H43" s="21" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="21" t="n"/>
+      <c r="K43" s="21" t="n"/>
+      <c r="L43" s="21" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8218,19 +8244,19 @@
         <v>0</v>
       </c>
       <c r="G46" s="8">
-        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <f>Premissas!$E$17/4*$D$45</f>
         <v/>
       </c>
       <c r="H46" s="8">
-        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <f>Premissas!$E$17/4*$D$45</f>
         <v/>
       </c>
       <c r="I46" s="8">
-        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <f>Premissas!$E$17/4*$D$45</f>
         <v/>
       </c>
       <c r="J46" s="8">
-        <f>Premissas!$E$17*Premissas!$E$18/4*$D$45</f>
+        <f>Premissas!$E$17/4*$D$45</f>
         <v/>
       </c>
       <c r="K46" s="8" t="n">
@@ -8352,13 +8378,13 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>-43876.1013425</v>
+        <v>-33799.9216625</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-11403.01613</v>
+        <v>16388.39815</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>63264.648615</v>
+        <v>114000.534375</v>
       </c>
     </row>
     <row r="9">
@@ -8406,7 +8432,7 @@
         <v>69825</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>237635</v>
+        <v>263927.5000000001</v>
       </c>
     </row>
     <row r="12">
@@ -8471,13 +8497,13 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>-43876.1013425</v>
+        <v>-33799.9216625</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>-11403.01613</v>
+        <v>16388.39815</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>63264.648615</v>
+        <v>114000.534375</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Aba de sensibilidade: efeito da chance de 1o lugar no cenario realista
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpMcBDEADLWoT4jSWTrqdN
</commit_message>
<xml_diff>
--- a/concursos/PROJECAO_CONCURSOS_2026_2028.xlsx
+++ b/concursos/PROJECAO_CONCURSOS_2026_2028.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realista" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otimista" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monte Carlo" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marcos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidade" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marcos" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -95,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -136,6 +137,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -8536,6 +8540,255 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>SENSIBILIDADE — e se a sua qualidade elevar a chance de 1º lugar? (cenário Realista, FIXO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Só a chance de 1º lugar por inscrição nacional muda (a de menção sobe junto, ~5× a do 1º). Inscrições, prêmios, contratos, margens e perna 2 ficam iguais ao Realista. 200 mil rodadas por linha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Chance de 1º por inscrição nacional</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Chance de menção</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Chance de pelo menos um 1º lugar em 2 anos</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Chance de pelo menos um contrato</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Caixa dos concursos — média</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Caixa — P10</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Caixa — P90</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Renda mensal média (com perna 2 do Realista)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="B5" s="27" t="n">
+        <v>0.1028</v>
+      </c>
+      <c r="C5" s="27" t="n">
+        <v>0.23109</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>0.103355</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>-11761.57535</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>-60480</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>15935</v>
+      </c>
+      <c r="H5" s="8">
+        <f>(E5+'Realista'!L35)/27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>0.1799</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>0.329775</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>0.17285</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>17115.521875</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>-53680</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>69825</v>
+      </c>
+      <c r="H6" s="8">
+        <f>(E6+'Realista'!L35)/27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>0.4188</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>0.241745</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46446.4801625</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>-46880</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>117310</v>
+      </c>
+      <c r="H7" s="8">
+        <f>(E7+'Realista'!L35)/27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>0.4112</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <v>0.565055</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>0.359185</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>104725.08405</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>-33280</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>175110</v>
+      </c>
+      <c r="H8" s="8">
+        <f>(E8+'Realista'!L35)/27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>0.70865</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>0.4921</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>174860.14095</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>-25375</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>262228.5000000005</v>
+      </c>
+      <c r="H9" s="8">
+        <f>(E9+'Realista'!L35)/27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="27" t="n">
+        <v>0.7843599999999999</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <v>0.570545</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>221538.3264</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>-19680</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>354005</v>
+      </c>
+      <c r="H10" s="8">
+        <f>(E10+'Realista'!L35)/27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Leitura: acima de ~8% por inscrição você estaria ganhando 1 em cada 12 concursos abertos. Isso é desempenho de escritório especialista com anos de histórico; não há dado seu para sustentar isso ainda.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8582,330 +8835,330 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>21/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Entrega UFC CACE</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="29" t="inlineStr">
         <is>
           <t>Maior valor esperado da carteira (contrato de R$ 7,24 mi de obra). Só aceita consórcio na inscrição.</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
+      <c r="D5" s="29" t="inlineStr">
         <is>
           <t>Edital</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>CAU do autor ativo (exigência do Sesc Carmo)</t>
         </is>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C6" s="29" t="inlineStr">
         <is>
           <t>Sem CAU ativo, o Sesc Carmo é desclassificado.</t>
         </is>
       </c>
-      <c r="D6" s="28" t="inlineStr">
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>Edital</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>11/11/2026</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Entrega Museu de Maringá</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
         <is>
           <t>Exige CNPJ e acervo CAT-A do vencedor.</t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr">
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>Edital</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>03/12/2026</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Sesc Carmo fase 1</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
         <is>
           <t>Líquido esperado levemente negativo; decisão é sua.</t>
         </is>
       </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>Edital</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>16/12/2026</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>House of Poetry</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
         <is>
           <t>Dezembro estoura o teto (200 h): tire um dos dois.</t>
         </is>
       </c>
-      <c r="D9" s="28" t="inlineStr">
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>Edital</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>até dez/2026</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Abrir o CNPJ da Djan Arquitetura</t>
         </is>
       </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
         <is>
           <t>Sem empresa, um 1º lugar pode virar só troféu. É o maior gargalo.</t>
         </is>
       </c>
-      <c r="D10" s="28" t="inlineStr">
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>Ação</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>até dez/2026</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>Definir acervo CAT-A: seu, de sócio ou de consórcio</t>
         </is>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
         <is>
           <t>Mesma razão: contrato público exige atestado de porte.</t>
         </is>
       </c>
-      <c r="D11" s="28" t="inlineStr">
+      <c r="D11" s="29" t="inlineStr">
         <is>
           <t>Ação</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>T1/2027</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>Resultados UFC e Maringá</t>
         </is>
       </c>
-      <c r="C12" s="28" t="inlineStr">
+      <c r="C12" s="29" t="inlineStr">
         <is>
           <t>Primeiro teste real do método. Qualquer resultado entra no portfólio.</t>
         </is>
       </c>
-      <c r="D12" s="28" t="inlineStr">
+      <c r="D12" s="29" t="inlineStr">
         <is>
           <t>Previsão</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>19/02/2027</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>Sassari</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>Só vale com parceiro italiano; com Unbuilt 2027 dá 315 h em fevereiro.</t>
         </is>
       </c>
-      <c r="D13" s="28" t="inlineStr">
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>Edital</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>4 a 6 nacionais com contrato, no máximo 1 grande por vez</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="29" t="inlineStr">
         <is>
           <t>Escalona a carga e concentra horas onde há contrato.</t>
         </is>
       </c>
-      <c r="D14" s="28" t="inlineStr">
+      <c r="D14" s="29" t="inlineStr">
         <is>
           <t>Estratégia</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>Cada concurso perdido vira peça de portfólio</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>Vitrine para cliente privado e para convites.</t>
         </is>
       </c>
-      <c r="D15" s="28" t="inlineStr">
+      <c r="D15" s="29" t="inlineStr">
         <is>
           <t>Estratégia</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>T3/2027</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>Primeiro contrato assinado (cenário realista)</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Dinheiro de contrato só chega ~3 trimestres após o resultado.</t>
         </is>
       </c>
-      <c r="D16" s="28" t="inlineStr">
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>Previsão</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="29" t="inlineStr">
         <is>
           <t>Execução de contrato disputa horas com concursos novos</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
+      <c r="C17" s="29" t="inlineStr">
         <is>
           <t>Contrato come ~300 h/trimestre; reduzir inscrições ou contratar apoio.</t>
         </is>
       </c>
-      <c r="D17" s="28" t="inlineStr">
+      <c r="D17" s="29" t="inlineStr">
         <is>
           <t>Estratégia</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>Convites para concursos fechados, júris e palestras</t>
         </is>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>Efeito de reputação, difícil de modelar; não entra na planilha.</t>
         </is>
       </c>
-      <c r="D18" s="28" t="inlineStr">
+      <c r="D18" s="29" t="inlineStr">
         <is>
           <t>Upside</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>dez/2028</t>
         </is>
       </c>
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="29" t="inlineStr">
         <is>
           <t>Balanço: carteira a receber, CNPJ, portfólio premiado</t>
         </is>
       </c>
-      <c r="C19" s="28" t="inlineStr">
+      <c r="C19" s="29" t="inlineStr">
         <is>
           <t>A linha 'carteira a receber após 2028' mostra o que já está ganho e ainda não pago.</t>
         </is>
       </c>
-      <c r="D19" s="28" t="inlineStr">
+      <c r="D19" s="29" t="inlineStr">
         <is>
           <t>Revisão</t>
         </is>

</xml_diff>